<commit_message>
feat: implement candidate search engine
</commit_message>
<xml_diff>
--- a/data/furniture.xlsx
+++ b/data/furniture.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E36F6A8B-3F09-412E-AF07-CDA19F143CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{98AB1377-DA10-4E8D-9E0C-6724EC958207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="293">
   <si>
     <t>Prompt 1</t>
   </si>
@@ -316,6 +316,9 @@
     <t>Poziom pewności</t>
   </si>
   <si>
+    <t>Search Features</t>
+  </si>
+  <si>
     <t>Fotel typ 366</t>
   </si>
   <si>
@@ -349,6 +352,9 @@
     <t>opracowania dotyczące Józefa Chierowskiego; dokumentacja 366 Concept; zbiory Muzeum Narodowego w Warszawie; Polski New Look Ewa Solarz i Agnieszka Sural; publikacje o polskim wzornictwie powojennym</t>
   </si>
   <si>
+    <t>drewniane boczki tworzące nogi i podłokietniki; trapezowe oparcie zwężające się ku górze; trapezowe siedzisko zwężające się ku tyłowi; widoczny prześwit pod siedziskiem; oddzielne moduły tapicerowanego siedziska i oparcia; skośnie rozstawione nogi; pozioma linia podłokietników; odsłonięte drewniane elementy boczne; lekka geometryczna bryła; brak tapicerowanych boków; zwężające się ku dołowi nogi; charakterystyczny profil boczny w kształcie odwróconego V</t>
+  </si>
+  <si>
     <t>Fotel typ 300-190</t>
   </si>
   <si>
@@ -376,6 +382,9 @@
     <t>Nowohuckie Renowacje – Fotel Lisek typ 300-190; Conchita Home – 4 fotele z PRL które musisz znać; dokumentacja i opisy egzemplarzy Typ 300-190; archiwalne materiały producentów cytowane w opracowaniach specjalistycznych</t>
   </si>
   <si>
+    <t>płaskie drewniane podłokietniki; toczone nogi zwężające się ku dołowi; nogi przechodzące przez podłokietniki; widoczna prostokątna rama boczna; poziome poprzeczki między nogami; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; smukła lekka bryła; odsłonięta konstrukcja drewniana; niskie podłokietniki; geometryczny profil boczny</t>
+  </si>
+  <si>
     <t>Do weryfikacji; często błędnie określany jako „Lisek”</t>
   </si>
   <si>
@@ -403,6 +412,9 @@
     <t>Patyna.pl – fotel B-7727 Radomsko PRL; Meblostan – fotel B-7727; Nowohuckie Renowacje – fotel B-7727; Vilandy – fotel Lis typ B-7727; Allegro – fotel PRL model B-7727 Radomsko lata 70; Reko-Czyny – identyfikacja fotela B-7727</t>
   </si>
   <si>
+    <t>otwarta drewniana rama boczna; prostokątne szerokie oparcie; oparcie szersze niż w modelu 300-190; prostokątne siedzisko; okrągłe toczone nogi; poziome drewniane podłokietniki; widoczne połączenia ramy bocznej; duży prześwit pod siedziskiem; lekka geometryczna bryła; drewniane belki łączące nogi; rozbieralne moduły siedziska i oparcia; nisko osadzone siedzisko</t>
+  </si>
+  <si>
     <t>Typ 300-177</t>
   </si>
   <si>
@@ -433,6 +445,9 @@
     <t>Meblostan – Fotel Bunny typ 300-177; Nowohuckie Renowacje – Fotel typ 300-177 Zajączek; Patyna.pl – Fotel Bunny typ 300-177; Tkaniny-Meblowe.pl – Fotele z PRL-u; materiały kolekcjonerskie rynku vintage</t>
   </si>
   <si>
+    <t>trójkątne podłokietniki przypominające uszy zająca; otwarta drewniana rama boczna; szeroko rozstawione nogi; podłokietniki połączone z przednimi nogami; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; smukła lekka bryła; odsłonięty drewniany stelaż; skośne tylne nogi; geometryczny profil boczny; kompaktowe proporcje</t>
+  </si>
+  <si>
     <t>Fotel Ewa; Muszelka Ewa</t>
   </si>
   <si>
@@ -457,6 +472,9 @@
     <t>Meblostan – Para foteli tapicerowanych EWA; Odnowa Mebli – Fotel Ewa; Patyna.pl – Komplet foteli typ Ewa; materiały kolekcjonerskie rynku vintage</t>
   </si>
   <si>
+    <t>muszelkowy korpus; kubełkowe siedzisko; zaokrąglone oparcie; stalowy stelaż; cztery smukłe metalowe nogi; wykręcane nogi; kulowe stopki; brak drewnianych podłokietników; jednolita tapicerowana bryła; szerokie półkoliste oparcie; lekka forma na wysokich nogach; profil przypominający muszlę</t>
+  </si>
+  <si>
     <t>Typ 300-123</t>
   </si>
   <si>
@@ -484,6 +502,9 @@
     <t>Nowohuckie Renowacje – Fotel typ 300-123 Puchała; Szajba Sklep – Fotel klubowy typ 300-123 proj. M. Puchała; LookInside – Fotel typ 300-123 Puchała; Pakamera – Fotel typ 300-123 M. Puchała; Meblostan – Fotel Puchały typ 300-123</t>
   </si>
   <si>
+    <t>gięte drewniane podłokietniki; smukłe wysokie oparcie; wąskie proporcje korpusu; otwarta drewniana rama boczna; toczone nogi zwężające się ku dołowi; widoczny prześwit pod siedziskiem; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; lekka dynamiczna bryła; cienkie elementy konstrukcyjne; profil boczny z łukowato wygiętym podłokietnikiem; minimalistyczna forma lat 50./60.</t>
+  </si>
+  <si>
     <t>RM58</t>
   </si>
   <si>
@@ -511,6 +532,9 @@
     <t>Muzeum Narodowe we Wrocławiu; Vzór – dokumentacja reedycji RM58; Instytut Wzornictwa Przemysłowego; publikacje o twórczości Romana Modzelewskiego; Culture.pl</t>
   </si>
   <si>
+    <t>jednoczęściowa muszelkowa skorupa; organiczna opływowa bryła; głębokie kubełkowe siedzisko; szerokie wywinięte boki; zaokrąglone wysokie oparcie; brak oddzielnych podłokietników; korpus przypominający muszlę; zamknięta forma boczna; cztery cienkie nogi; futurystyczna sylwetka lat 50.; brak widocznej drewnianej konstrukcji; płynne przejścia między siedziskiem i oparciem; asymetrycznie zaokrąglone krawędzie; korpus wykonany jako pojedyncza skorupa</t>
+  </si>
+  <si>
     <t>B-2020</t>
   </si>
   <si>
@@ -541,6 +565,9 @@
     <t>FAMEG – Fotel Tulipan B-2020; dokumentacja reedycji FAMEG; opracowania dotyczące twórczości Teresy Kruszewskiej</t>
   </si>
   <si>
+    <t>kubełkowe siedzisko; forma przypominająca kielich tulipana; szeroko rozchylone boki; jednolita tapicerowana skorupa; zaokrąglone wysokie oparcie; płynne przejście między siedziskiem i oparciem; organiczna bryła; brak widocznej drewnianej ramy bocznej; miękkie obłe krawędzie; rzeźbiarska forma; kompaktowa podstawa; sylwetka kwiatu tulipana</t>
+  </si>
+  <si>
     <t>Typ 300-201</t>
   </si>
   <si>
@@ -566,368 +593,338 @@
   </si>
   <si>
     <t>Meblostan – Fotel Śnieżnik typ 300-201; Nowohuckie Renowacje – Fotele PRL; Pakamera – Fotel Śnieżnik typ 300-201; Audiovintage Store – Fotel klubowy Śnieżnik 300-201</t>
-  </si>
-  <si>
-    <t>GFM-57</t>
-  </si>
-  <si>
-    <t>Skoczek</t>
-  </si>
-  <si>
-    <t>Juliusz Kędziorek</t>
-  </si>
-  <si>
-    <t>Krzesło</t>
-  </si>
-  <si>
-    <t>Gościcińska Fabryka Mebli; Zamojskie Fabryki Mebli (produkcja seryjna jako typ 200-203)</t>
-  </si>
-  <si>
-    <t>łukowate podłokietniki przypominające profil skoczni narciarskiej; elipsoidalne oparcie; lekka ażurowa konstrukcja; zwężające się ku dołowi nogi; tapicerowane siedzisko; smukła sylwetka; organiczna linia boczna</t>
-  </si>
-  <si>
-    <t>drewniany stelaż; otwarta konstrukcja boczna; tapicerowane siedzisko; gięte elementy drewniane; konstrukcja przeznaczona do produkcji seryjnej</t>
-  </si>
-  <si>
-    <t>typ 200-190 Rajmunda Hałasa; krzesła Aga; krzesła patyczaki lat 60.; lekkie krzesła tapicerowane PRL</t>
-  </si>
-  <si>
-    <t>typ 200-203; GFM-107; projekty Juliusza Kędziorka dla Gościcińskiej Fabryki Mebli</t>
-  </si>
-  <si>
-    <t>Magazif – Krzesło Skoczek; Ikony Designu PL – Krzesło GFM-57 Skoczek; Meblostan – Krzesło Skoczek; Sosenko Home Decor – Krzesło Skoczek; Allegro Artykuł – Krzesło kilka słów o najtrudniejszym meblu</t>
-  </si>
-  <si>
-    <t>Typ 200-125 VAR</t>
-  </si>
-  <si>
-    <t>Aga</t>
-  </si>
-  <si>
-    <t>ok. 1972–1975 (w źródłach występują rozbieżności dotyczące dokładnego roku projektu)</t>
-  </si>
-  <si>
-    <t>Wielkopolskie Fabryki Mebli; produkcja seryjna PRL (pozostali producenci wymagają weryfikacji)</t>
-  </si>
-  <si>
-    <t>wysokie tapicerowane oparcie; trapezowy układ nóg; miękkie tapicerowane siedzisko; smukła skandynawska forma; zwężająca się ku górze bryła; lekkie proporcje; drewniana konstrukcja eksponowana po bokach</t>
-  </si>
-  <si>
-    <t>drewniany stelaż bukowy; tapicerowane siedzisko; tapicerowane oparcie; sprężyny siedziska; cztery drewniane nogi; konstrukcja przeznaczona do intensywnego użytkowania klubowego</t>
-  </si>
-  <si>
-    <t>typ 200-190 Rajmunda Hałasa; GFM-57 Skoczek; lekkie krzesła klubowe PRL lat 70.</t>
-  </si>
-  <si>
-    <t>fotel 366; meble klubowe Józefa Chierowskiego; reedycja 200-125 VAR realizowana przez 366 Concept</t>
-  </si>
-  <si>
-    <t>Elle Decoration Polska – Krzesło VAR AGA projektu Józefa Chierowskiego; Nowohuckie Renowacje – Krzesło Aga typ 200-125; Patyna.pl – Krzesła AGA typu 200-125 VAR; Linie Studio – 200-125 VAR; Meblościanka – 200-125 VAR</t>
-  </si>
-  <si>
-    <t>Typ 200-190</t>
-  </si>
-  <si>
-    <t>Hałas; Grzybek</t>
-  </si>
-  <si>
-    <t>Rajmund Teofil Hałas</t>
-  </si>
-  <si>
-    <t>lata 60. XX w.; dokładny rok projektu – Do weryfikacji</t>
-  </si>
-  <si>
-    <t>Zakłady Mebli w Gostyniu (Do weryfikacji); produkcja seryjna w kilku zakładach meblarskich PRL – Do weryfikacji</t>
-  </si>
-  <si>
-    <t>okrągła forma oparcia przypominająca kapelusz grzyba; tapicerowane oparcie i siedzisko; smukłe zwężające się nogi; lekka konstrukcja; wyraźnie wyodrębnione oparcie nad siedziskiem; proporcje inspirowane wzornictwem skandynawskim; minimalistyczna sylwetka</t>
-  </si>
-  <si>
-    <t>drewniany stelaż; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; mocowane oddzielnie siedzisko i oparcie; nogi zwężające się ku dołowi</t>
-  </si>
-  <si>
-    <t>Aga 200-125; Skoczek GFM-57; krzesła skandynawskie lat 60.; lekkie krzesła tapicerowane PRL</t>
-  </si>
-  <si>
-    <t>projekty Rajmunda Teofila Hałasa; krzesła tapicerowane PRL lat 60.; warianty produkcyjne typu 200-190</t>
-  </si>
-  <si>
-    <t>Odnawialnia – Wiem co odnawiam | krzesło Hałasa typ 200-190; Patyna.pl – Krzesła typ 200-190 Rajmund Teofil Hałas; Meblostan – Komplet krzeseł typ 200-190; Daniel Stoiński Redesign – Przewodnik po renowacji krzesła 200-190; Homebook – Krzesło Hałasa typ 200-190</t>
-  </si>
-  <si>
-    <t>B-6028</t>
-  </si>
-  <si>
-    <t>Barbara Fenrych-Węcławska (Do weryfikacji); Józef Chierowski (Do weryfikacji – atrybucja pojawiająca się wyłącznie w źródłach kolekcjonerskich)</t>
-  </si>
-  <si>
-    <t>lata 60. XX w.</t>
-  </si>
-  <si>
-    <t>Fabryka Mebli Giętych w Radomsku; FAMEG Radomsko; Radomszczańska Fabryka Mebli Giętych</t>
-  </si>
-  <si>
-    <t>wysokie profilowane oparcie; szerokie drewniane podłokietniki; gięte elementy bukowe; głębokie siedzisko; lekka otwarta konstrukcja boczna; elegancka smukła sylwetka; forma łącząca cechy fotela klubowego i wypoczynkowego</t>
-  </si>
-  <si>
-    <t>stelaż z giętego drewna bukowego; otwarta konstrukcja ramowa; tapicerowane siedzisko; tapicerowane oparcie; drewniane podłokietniki zintegrowane z ramą; konstrukcja szkieletowa</t>
-  </si>
-  <si>
-    <t>typ 300-123 Puchała; typ 300-177 Zajączek; B-7727; typ 366</t>
-  </si>
-  <si>
-    <t>fotele Radomsko z giętego drewna; projekty Barbary Fenrych-Węcławskiej (Do weryfikacji); lekkie fotele klubowe PRL lat 60.</t>
-  </si>
-  <si>
-    <t>MidMod – Fotel B6028 FAMEG Radomsko Polska lata 60; Oldsen Design – Fotel B6028 prod. FAMEG Radomsko; Nowohuckie Renowacje – Fotel PRL B-6028 z lat 60-tych; Fotelowo Facebook – fotel projektu Barbary Fenrych-Węcławskiej; Instagram Renowacja Mebli PRL – B6028 lata produkcji 1960</t>
-  </si>
-  <si>
-    <t>A. Dutka</t>
-  </si>
-  <si>
-    <t>1966–1968</t>
-  </si>
-  <si>
-    <t>Zakłady Mebli Giętych w Radomsku; Gołuchowskie Fabryki Mebli</t>
-  </si>
-  <si>
-    <t>duże gabaryty; szerokie głębokie siedzisko; masywne drewniane podłokietniki; geometryczna forma boczna; lekko pochylone oparcie; otwarta konstrukcja ramowa; modernistyczna sylwetka eksportowa</t>
-  </si>
-  <si>
-    <t>stelaż z drewna bukowego; sprężyny lejowe w siedzisku; tapicerowane siedzisko i oparcie; otwarta konstrukcja boczna; drewniane podłokietniki zintegrowane z ramą; konstrukcja rozbieralna skręcana śrubami</t>
-  </si>
-  <si>
-    <t>B-6028; GFM-64; typ 300-190 Lisek; B-7727</t>
-  </si>
-  <si>
-    <t>fotele eksportowe Radomsko lat 60.; modele Zakładów Mebli Giętych w Radomsku; konstrukcje projektowane przez A. Dutkę (Do weryfikacji)</t>
-  </si>
-  <si>
-    <t>Meblostan – Para foteli B-310 VAR; Pufa Design – Oryginalny fotel B-310 VAR; Yestersen – Fotel B-310 VAR Polska lata 70.; Reko-Czyny – Fotel B-310 VAR metamorfoza; archiwalne ogłoszenia kolekcjonerskie B-310 VAR</t>
-  </si>
-  <si>
-    <t>GFM-22 (typ 200/128)</t>
-  </si>
-  <si>
-    <t>ok. 1960</t>
-  </si>
-  <si>
-    <t>Gościcińska Fabryka Mebli (GFM)</t>
-  </si>
-  <si>
-    <t>nerkowate oparcie; lekka ażurowa konstrukcja; smukłe zwężające się nogi; gięta drewniana rama; tapicerowane siedzisko; tapicerowane oparcie; wyraźnie rozstawione tylne nogi</t>
-  </si>
-  <si>
-    <t>drewniany stelaż; gięte elementy z litego drewna; tapicerowane siedzisko; tapicerowane oparcie ze sklejki giętej; konstrukcja szkieletowa przeznaczona do produkcji seryjnej</t>
-  </si>
-  <si>
-    <t>GFM-57 Skoczek; typ 200-190 Rajmunda Hałasa; Aga 200-125; krzesła skandynawskie z lat 60.</t>
-  </si>
-  <si>
-    <t>typ 200/128; projekty Juliusza Kędziorka dla Gościcińskiej Fabryki Mebli; GFM-57; GFM-87</t>
-  </si>
-  <si>
-    <t>Pamono – Mid-Century GFM-22 Chairs by Juliusz Kędziorek; Vinterior – GFM-22 model 200/128; Selency – Iconic GFM-22 Chair by Juliusz Kędziorek; Instagram Zostań z Vintage – Krzesło GFM-22 typ 200/128</t>
-  </si>
-  <si>
-    <t>Typ 1020</t>
-  </si>
-  <si>
-    <t>Muszelka</t>
-  </si>
-  <si>
-    <t>Wiesław Leśniewski; Stanisław Lejkowski</t>
-  </si>
-  <si>
-    <t>Słupskie Fabryki Mebli</t>
-  </si>
-  <si>
-    <t>muszelkowe profilowane oparcie; jednolita tapicerowana skorupa; zaokrąglona górna krawędź oparcia; smukłe stożkowe nogi; lekka modernistyczna forma; brak podłokietników; organiczna sylwetka</t>
-  </si>
-  <si>
-    <t>profilowana skorupa ze sklejki; tapicerowana skorupa; drewniany stelaż; cztery drewniane nogi; konstrukcja szkieletowa; połączenie sklejki i drewna litego</t>
-  </si>
-  <si>
-    <t>RM58; krzesła muszelkowe produkcji NRD; krzesła skandynawskie lat 60.; fotel Ewa</t>
-  </si>
-  <si>
-    <t>krzesła muszelkowe Słupskich Fabryk Mebli; projekty Wiesława Leśniewskiego i Stanisława Lejkowskiego; meble ze sklejki profilowanej produkowane przez SFM</t>
-  </si>
-  <si>
-    <t>Archiwalne katalogi Słupskich Fabryk Mebli; opracowania kolekcjonerskie dotyczące wzornictwa SFM; materiały renowatorów specjalizujących się w meblach PRL; publikacje poświęcone projektom Wiesława Leśniewskiego i Stanisława Lejkowskiego</t>
-  </si>
-  <si>
-    <t>Bumerang</t>
-  </si>
-  <si>
-    <t>Ryszard Kulm</t>
-  </si>
-  <si>
-    <t>przełom lat 50. i 60. XX w.; produkcja seryjna od początku lat 60</t>
-  </si>
-  <si>
-    <t>Gościcińska Fabryka Mebli</t>
-  </si>
-  <si>
-    <t>charakterystyczne łukowato wygięte przednie nogi przypominające bumerang; lekka ażurowa konstrukcja; tapicerowane siedzisko; tapicerowane oparcie; smukła sylwetka; zwężające się ku dołowi nogi; modernistyczna forma inspirowana skandynawskim wzornictwem</t>
-  </si>
-  <si>
-    <t>drewniany stelaż bukowy; gięte elementy boczne; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; połączenia skręcane i klejone</t>
-  </si>
-  <si>
-    <t>GFM-22; typ 200-190 Rajmunda Hałasa; GFM-57 Skoczek; krzesła skandynawskie lat 60</t>
-  </si>
-  <si>
-    <t>krzesła Gościcińskiej Fabryki Mebli; wariant 299XB (Do weryfikacji); rodzina krzeseł Bumerang</t>
-  </si>
-  <si>
-    <t>Meblostan – Komplet 4 krzeseł Bumerang typ 299; Skarby PRL – Krzesło tapicerowane Bumerang typ 299; Patyna – Komplet krzeseł typ 299 Bumerang; Deccoria – 10 słynnych mebli z PRL; Stary Fotel – Krzesła Bumerang metamorfoza</t>
-  </si>
-  <si>
-    <t>Typ 300-227</t>
-  </si>
-  <si>
-    <t>Celia</t>
-  </si>
-  <si>
-    <t>ok. 1965; produkcja na przełomie lat 60. i 70. XX w.</t>
-  </si>
-  <si>
-    <t>Zamojskie Fabryki Mebli</t>
-  </si>
-  <si>
-    <t>brak podłokietników; toczone drewniane nogi umieszczone po bokach części tapicerowanej; trapezowe siedzisko; proste tapicerowane oparcie; lekka minimalistyczna forma; kompaktowe wymiary; stylistyka skandynawskiego modernizmu</t>
-  </si>
-  <si>
-    <t>drewniany stelaż; toczone nogi; tapicerowane siedzisko; tapicerowane oparcie; otwarta konstrukcja bez podłokietników; konstrukcja szkieletowa przeznaczona do produkcji seryjnej</t>
-  </si>
-  <si>
-    <t>typ 300-190 Lisek; typ 366; GFM-64; lekkie fotele klubowe PRL bez podłokietników</t>
-  </si>
-  <si>
-    <t>fotele Zamojskich Fabryk Mebli z lat 60. i 70.; meble klubowe produkowane w Zamościu; modele o minimalistycznej konstrukcji bez podłokietników</t>
-  </si>
-  <si>
-    <t>Meblostan – Fotel CELIA typ 300-227; Patyna – Fotel CELIA typ 300-227 PRL; Szajba Sklep – Fotel Celia typ 300-227; materiały kolekcjonerskie dotyczące Zamojskich Fabryk Mebli</t>
-  </si>
-  <si>
-    <t>Typ 300-139</t>
-  </si>
-  <si>
-    <t>Stefan</t>
-  </si>
-  <si>
-    <t>Swarzędzka Fabryka Mebli</t>
-  </si>
-  <si>
-    <t>szerokie drewniane podłokietniki o łagodnym łuku; otwarta konstrukcja boczna; luźne tapicerowane poduchy siedziska i oparcia; rozłożysta bryła; lekka skandynawska stylistyka; nisko osadzone siedzisko; masywny drewniany stelaż</t>
-  </si>
-  <si>
-    <t>stelaż z litego drewna bukowego; otwarta rama boczna; osobna poduszka siedziska; osobna poduszka oparcia; pasy tapicerskie; konstrukcja szkieletowa skręcana</t>
-  </si>
-  <si>
-    <t>typ 300-123 Puchała; typ 366; duńskie fotele Kandidaten projektu Ib Kofod-Larsena; fotele skandynawskie lat 60</t>
-  </si>
-  <si>
-    <t>sofa Stefan; zestawy wypoczynkowe Swarzędzkiej Fabryki Mebli; meble eksportowe Swarzędzkiej Fabryki Mebli z lat 60.</t>
-  </si>
-  <si>
-    <t>„Meble w produkcji 1962” – Zjednoczenie Przemysłu Meblarskiego; „Meble do małych mieszkań. Informator”, Wydawnictwo Katalogów i Cenników 1966; Laminerva – „Ikony polskiego designu: Fotel Stefan typ 300-139”; Meblostan – Para foteli Stefan typ 300-139; Patyna – Para foteli Stefan typ 300-139</t>
-  </si>
-  <si>
-    <t>B-3300</t>
-  </si>
-  <si>
-    <t>ok. 1969; produkcja w końcu lat 60. i na początku lat 70. XX w</t>
-  </si>
-  <si>
-    <t>Zakład Mebli Giętych w Radomsku; Fabryki Mebli Radomsko (późniejsze nazewnictwo zakładu)</t>
-  </si>
-  <si>
-    <t>gięte drewniane podłokietniki; szerokie tapicerowane siedzisko; prostokątne tapicerowane oparcie; otwarta konstrukcja boczna; gięty bukowy stelaż; nisko osadzona bryła; elegancka modernistyczna forma</t>
-  </si>
-  <si>
-    <t>stelaż z giętego drewna bukowego; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; elementy gięte wykonane w technologii Thoneta; konstrukcja skręcana</t>
-  </si>
-  <si>
-    <t>B-310 VAR; B-6028; GFM-64; typ 300-139 Stefan</t>
-  </si>
-  <si>
-    <t>fotele Zakładu Mebli Giętych w Radomsku; modele eksportowe Radomsko z lat 60. i 70.; rodzina foteli z giętego drewna bukowego</t>
-  </si>
-  <si>
-    <t>Patyna – Fotel B-3300 Zakład Mebli Giętych w Radomsku; Meblostan – Para foteli B-3300; archiwalne materiały Fabryk Mebli Radomsko; oferty kolekcjonerskie dokumentujące oryginalne oznaczenie modelu</t>
-  </si>
-  <si>
-    <t>Cechy AI</t>
-  </si>
-  <si>
-    <t>drewniane boczki tworzące nogi i podłokietniki; trapezowe oparcie zwężające się ku górze; trapezowe siedzisko zwężające się ku tyłowi; widoczny prześwit pod siedziskiem; oddzielne moduły tapicerowanego siedziska i oparcia; skośnie rozstawione nogi; pozioma linia podłokietników; odsłonięte drewniane elementy boczne; lekka geometryczna bryła; brak tapicerowanych boków; zwężające się ku dołowi nogi; charakterystyczny profil boczny w kształcie odwróconego V</t>
-  </si>
-  <si>
-    <t>Typ 300-190</t>
-  </si>
-  <si>
-    <t>płaskie drewniane podłokietniki; toczone nogi zwężające się ku dołowi; nogi przechodzące przez podłokietniki; widoczna prostokątna rama boczna; poziome poprzeczki między nogami; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; smukła lekka bryła; odsłonięta konstrukcja drewniana; niskie podłokietniki; geometryczny profil boczny</t>
-  </si>
-  <si>
-    <t>otwarta drewniana rama boczna; prostokątne szerokie oparcie; oparcie szersze niż w modelu 300-190; prostokątne siedzisko; okrągłe toczone nogi; poziome drewniane podłokietniki; widoczne połączenia ramy bocznej; duży prześwit pod siedziskiem; lekka geometryczna bryła; drewniane belki łączące nogi; rozbieralne moduły siedziska i oparcia; nisko osadzone siedzisko</t>
-  </si>
-  <si>
-    <t>trójkątne podłokietniki przypominające uszy zająca; otwarta drewniana rama boczna; szeroko rozstawione nogi; podłokietniki połączone z przednimi nogami; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; smukła lekka bryła; odsłonięty drewniany stelaż; skośne tylne nogi; geometryczny profil boczny; kompaktowe proporcje</t>
-  </si>
-  <si>
-    <t>muszelkowy korpus; kubełkowe siedzisko; zaokrąglone oparcie; stalowy stelaż; cztery smukłe metalowe nogi; wykręcane nogi; kulowe stopki; brak drewnianych podłokietników; jednolita tapicerowana bryła; szerokie półkoliste oparcie; lekka forma na wysokich nogach; profil przypominający muszlę</t>
-  </si>
-  <si>
-    <t>gięte drewniane podłokietniki; smukłe wysokie oparcie; wąskie proporcje korpusu; otwarta drewniana rama boczna; toczone nogi zwężające się ku dołowi; widoczny prześwit pod siedziskiem; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; lekka dynamiczna bryła; cienkie elementy konstrukcyjne; profil boczny z łukowato wygiętym podłokietnikiem; minimalistyczna forma lat 50./60.</t>
-  </si>
-  <si>
-    <t>jednoczęściowa muszelkowa skorupa; organiczna opływowa bryła; głębokie kubełkowe siedzisko; szerokie wywinięte boki; zaokrąglone wysokie oparcie; brak oddzielnych podłokietników; korpus przypominający muszlę; zamknięta forma boczna; cztery cienkie nogi; futurystyczna sylwetka lat 50.; brak widocznej drewnianej konstrukcji; płynne przejścia między siedziskiem i oparciem; asymetrycznie zaokrąglone krawędzie; korpus wykonany jako pojedyncza skorupa</t>
-  </si>
-  <si>
-    <t>kubełkowe siedzisko; forma przypominająca kielich tulipana; szeroko rozchylone boki; jednolita tapicerowana skorupa; zaokrąglone wysokie oparcie; płynne przejście między siedziskiem i oparciem; organiczna bryła; brak widocznej drewnianej ramy bocznej; miękkie obłe krawędzie; rzeźbiarska forma; kompaktowa podstawa; sylwetka kwiatu tulipana</t>
   </si>
   <si>
     <t>otwarta drewniana rama boczna; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; smukła lekka bryła; duży prześwit pod siedziskiem; drewniane podłokietniki zintegrowane z ramą; nogi graniaste od góry; nogi zaokrąglone w dolnej części; skośne tylne nogi; widoczne drewniane elementy konstrukcyjne; forma zbliżona do modelu Lisek; geometryczny profil boczny
 Źródła potwierdzają produkcję w Bystrzyckiej Fabryce Mebli oraz silne pokrewieństwo konstrukcyjne z modelem 300-190 „Lisek”, natomiast projektant pozostaje niepotwierdzony.</t>
   </si>
   <si>
-    <t>GFM-57 Skoczek</t>
+    <t>GFM-57</t>
+  </si>
+  <si>
+    <t>Skoczek</t>
+  </si>
+  <si>
+    <t>Juliusz Kędziorek</t>
+  </si>
+  <si>
+    <t>Krzesło</t>
+  </si>
+  <si>
+    <t>Gościcińska Fabryka Mebli; Zamojskie Fabryki Mebli (produkcja seryjna jako typ 200-203)</t>
+  </si>
+  <si>
+    <t>łukowate podłokietniki przypominające profil skoczni narciarskiej; elipsoidalne oparcie; lekka ażurowa konstrukcja; zwężające się ku dołowi nogi; tapicerowane siedzisko; smukła sylwetka; organiczna linia boczna</t>
+  </si>
+  <si>
+    <t>drewniany stelaż; otwarta konstrukcja boczna; tapicerowane siedzisko; gięte elementy drewniane; konstrukcja przeznaczona do produkcji seryjnej</t>
+  </si>
+  <si>
+    <t>typ 200-190 Rajmunda Hałasa; krzesła Aga; krzesła patyczaki lat 60.; lekkie krzesła tapicerowane PRL</t>
+  </si>
+  <si>
+    <t>typ 200-203; GFM-107; projekty Juliusza Kędziorka dla Gościcińskiej Fabryki Mebli</t>
+  </si>
+  <si>
+    <t>Magazif – Krzesło Skoczek; Ikony Designu PL – Krzesło GFM-57 Skoczek; Meblostan – Krzesło Skoczek; Sosenko Home Decor – Krzesło Skoczek; Allegro Artykuł – Krzesło kilka słów o najtrudniejszym meblu</t>
   </si>
   <si>
     <t>łukowate podłokietniki przypominające skocznię narciarską; elipsoidalne oparcie; otwarta drewniana rama boczna; smukłe zwężające się nogi; tapicerowane siedzisko; duży prześwit pod siedziskiem; płynna linia podłokietnika przechodząca w nogę; lekka ażurowa konstrukcja; organiczny profil boczny; oparcie w kształcie pionowej elipsy; cienkie elementy drewniane; dynamiczna sylwetka inspirowana skokami narciarskimi
 Źródła potwierdzają, że model został zaprojektowany przez Juliusza Kędziorka w Gościcińskiej Fabryce Mebli w 1965 r., otrzymał nagrodę „Dobre–Ładne–Poszukiwane” i został skierowany do produkcji seryjnej jako typ 200-203</t>
   </si>
   <si>
+    <t>Typ 200-125 VAR</t>
+  </si>
+  <si>
+    <t>Aga</t>
+  </si>
+  <si>
+    <t>ok. 1972–1975 (w źródłach występują rozbieżności dotyczące dokładnego roku projektu)</t>
+  </si>
+  <si>
+    <t>Wielkopolskie Fabryki Mebli; produkcja seryjna PRL (pozostali producenci wymagają weryfikacji)</t>
+  </si>
+  <si>
+    <t>wysokie tapicerowane oparcie; trapezowy układ nóg; miękkie tapicerowane siedzisko; smukła skandynawska forma; zwężająca się ku górze bryła; lekkie proporcje; drewniana konstrukcja eksponowana po bokach</t>
+  </si>
+  <si>
+    <t>drewniany stelaż bukowy; tapicerowane siedzisko; tapicerowane oparcie; sprężyny siedziska; cztery drewniane nogi; konstrukcja przeznaczona do intensywnego użytkowania klubowego</t>
+  </si>
+  <si>
+    <t>typ 200-190 Rajmunda Hałasa; GFM-57 Skoczek; lekkie krzesła klubowe PRL lat 70.</t>
+  </si>
+  <si>
+    <t>fotel 366; meble klubowe Józefa Chierowskiego; reedycja 200-125 VAR realizowana przez 366 Concept</t>
+  </si>
+  <si>
+    <t>Elle Decoration Polska – Krzesło VAR AGA projektu Józefa Chierowskiego; Nowohuckie Renowacje – Krzesło Aga typ 200-125; Patyna.pl – Krzesła AGA typu 200-125 VAR; Linie Studio – 200-125 VAR; Meblościanka – 200-125 VAR</t>
+  </si>
+  <si>
     <t>wysokie tapicerowane oparcie; trapezowy układ nóg; szerokie miękkie siedzisko; brak podłokietników; drewniane nogi rozszerzające się ku dołowi; zwężająca się ku górze sylwetka; lekka skandynawska forma; prostokątne oparcie z zaokrąglonymi krawędziami; widoczne drewniane elementy boczne; smukłe proporcje; geometryczna bryła; profil boczny z pochylonym oparciem</t>
   </si>
   <si>
+    <t>Typ 200-190</t>
+  </si>
+  <si>
+    <t>Hałas; Grzybek</t>
+  </si>
+  <si>
+    <t>Rajmund Teofil Hałas</t>
+  </si>
+  <si>
+    <t>lata 60. XX w.; dokładny rok projektu – Do weryfikacji</t>
+  </si>
+  <si>
+    <t>Zakłady Mebli w Gostyniu (Do weryfikacji); produkcja seryjna w kilku zakładach meblarskich PRL – Do weryfikacji</t>
+  </si>
+  <si>
+    <t>okrągła forma oparcia przypominająca kapelusz grzyba; tapicerowane oparcie i siedzisko; smukłe zwężające się nogi; lekka konstrukcja; wyraźnie wyodrębnione oparcie nad siedziskiem; proporcje inspirowane wzornictwem skandynawskim; minimalistyczna sylwetka</t>
+  </si>
+  <si>
+    <t>drewniany stelaż; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; mocowane oddzielnie siedzisko i oparcie; nogi zwężające się ku dołowi</t>
+  </si>
+  <si>
+    <t>Aga 200-125; Skoczek GFM-57; krzesła skandynawskie lat 60.; lekkie krzesła tapicerowane PRL</t>
+  </si>
+  <si>
+    <t>projekty Rajmunda Teofila Hałasa; krzesła tapicerowane PRL lat 60.; warianty produkcyjne typu 200-190</t>
+  </si>
+  <si>
+    <t>Odnawialnia – Wiem co odnawiam | krzesło Hałasa typ 200-190; Patyna.pl – Krzesła typ 200-190 Rajmund Teofil Hałas; Meblostan – Komplet krzeseł typ 200-190; Daniel Stoiński Redesign – Przewodnik po renowacji krzesła 200-190; Homebook – Krzesło Hałasa typ 200-190</t>
+  </si>
+  <si>
     <t>okrągłe oparcie przypominające grzybek; oparcie szersze od wspornika; tapicerowane okrągłe oparcie; tapicerowane siedzisko; smukłe nogi zwężające się ku dołowi; brak podłokietników; lekka skandynawska forma; duży prześwit pod siedziskiem; cienki drewniany stelaż; wyraźne oddzielenie oparcia od siedziska; geometryczna bryła; profil boczny z lekko odchylonym oparciem</t>
   </si>
   <si>
+    <t>B-6028</t>
+  </si>
+  <si>
+    <t>Barbara Fenrych-Węcławska (Do weryfikacji); Józef Chierowski (Do weryfikacji – atrybucja pojawiająca się wyłącznie w źródłach kolekcjonerskich)</t>
+  </si>
+  <si>
+    <t>lata 60. XX w.</t>
+  </si>
+  <si>
+    <t>Fabryka Mebli Giętych w Radomsku; FAMEG Radomsko; Radomszczańska Fabryka Mebli Giętych</t>
+  </si>
+  <si>
+    <t>wysokie profilowane oparcie; szerokie drewniane podłokietniki; gięte elementy bukowe; głębokie siedzisko; lekka otwarta konstrukcja boczna; elegancka smukła sylwetka; forma łącząca cechy fotela klubowego i wypoczynkowego</t>
+  </si>
+  <si>
+    <t>stelaż z giętego drewna bukowego; otwarta konstrukcja ramowa; tapicerowane siedzisko; tapicerowane oparcie; drewniane podłokietniki zintegrowane z ramą; konstrukcja szkieletowa</t>
+  </si>
+  <si>
+    <t>typ 300-123 Puchała; typ 300-177 Zajączek; B-7727; typ 366</t>
+  </si>
+  <si>
+    <t>fotele Radomsko z giętego drewna; projekty Barbary Fenrych-Węcławskiej (Do weryfikacji); lekkie fotele klubowe PRL lat 60.</t>
+  </si>
+  <si>
+    <t>MidMod – Fotel B6028 FAMEG Radomsko Polska lata 60; Oldsen Design – Fotel B6028 prod. FAMEG Radomsko; Nowohuckie Renowacje – Fotel PRL B-6028 z lat 60-tych; Fotelowo Facebook – fotel projektu Barbary Fenrych-Węcławskiej; Instagram Renowacja Mebli PRL – B6028 lata produkcji 1960</t>
+  </si>
+  <si>
     <t>wysokie prostokątne oparcie; szerokie drewniane podłokietniki; gięte boczne elementy z drewna; otwarta rama boczna; głębokie siedzisko; masywniejsza bryła niż typ 366; bukowy stelaż; duży prześwit pod siedziskiem; profilowane podłokietniki; smukłe nogi zintegrowane z ramą; tapicerowane oparcie i siedzisko; geometryczny profil boczny</t>
   </si>
   <si>
+    <t>A. Dutka</t>
+  </si>
+  <si>
+    <t>1966–1968</t>
+  </si>
+  <si>
+    <t>Zakłady Mebli Giętych w Radomsku; Gołuchowskie Fabryki Mebli</t>
+  </si>
+  <si>
+    <t>duże gabaryty; szerokie głębokie siedzisko; masywne drewniane podłokietniki; geometryczna forma boczna; lekko pochylone oparcie; otwarta konstrukcja ramowa; modernistyczna sylwetka eksportowa</t>
+  </si>
+  <si>
+    <t>stelaż z drewna bukowego; sprężyny lejowe w siedzisku; tapicerowane siedzisko i oparcie; otwarta konstrukcja boczna; drewniane podłokietniki zintegrowane z ramą; konstrukcja rozbieralna skręcana śrubami</t>
+  </si>
+  <si>
+    <t>B-6028; GFM-64; typ 300-190 Lisek; B-7727</t>
+  </si>
+  <si>
+    <t>fotele eksportowe Radomsko lat 60.; modele Zakładów Mebli Giętych w Radomsku; konstrukcje projektowane przez A. Dutkę (Do weryfikacji)</t>
+  </si>
+  <si>
+    <t>Meblostan – Para foteli B-310 VAR; Pufa Design – Oryginalny fotel B-310 VAR; Yestersen – Fotel B-310 VAR Polska lata 70.; Reko-Czyny – Fotel B-310 VAR metamorfoza; archiwalne ogłoszenia kolekcjonerskie B-310 VAR</t>
+  </si>
+  <si>
     <t>masywne drewniane podłokietniki; szerokie głębokie siedzisko; wysunięte przednie podłokietniki; otwarta drewniana rama boczna; prostokątne tapicerowane oparcie; grube proporcje siedziska; lekko pochylone oparcie; duży prześwit pod siedziskiem; widoczne śruby montażowe w ramie; geometryczny profil boczny; szeroki rozstaw nóg; cięższa bryła niż typ 366; bukowy stelaż; modernistyczna forma eksportowa</t>
   </si>
   <si>
+    <t>GFM-22 (typ 200/128)</t>
+  </si>
+  <si>
+    <t>ok. 1960</t>
+  </si>
+  <si>
+    <t>Gościcińska Fabryka Mebli (GFM)</t>
+  </si>
+  <si>
+    <t>nerkowate oparcie; lekka ażurowa konstrukcja; smukłe zwężające się nogi; gięta drewniana rama; tapicerowane siedzisko; tapicerowane oparcie; wyraźnie rozstawione tylne nogi</t>
+  </si>
+  <si>
+    <t>drewniany stelaż; gięte elementy z litego drewna; tapicerowane siedzisko; tapicerowane oparcie ze sklejki giętej; konstrukcja szkieletowa przeznaczona do produkcji seryjnej</t>
+  </si>
+  <si>
+    <t>GFM-57 Skoczek; typ 200-190 Rajmunda Hałasa; Aga 200-125; krzesła skandynawskie z lat 60.</t>
+  </si>
+  <si>
+    <t>typ 200/128; projekty Juliusza Kędziorka dla Gościcińskiej Fabryki Mebli; GFM-57; GFM-87</t>
+  </si>
+  <si>
+    <t>Pamono – Mid-Century GFM-22 Chairs by Juliusz Kędziorek; Vinterior – GFM-22 model 200/128; Selency – Iconic GFM-22 Chair by Juliusz Kędziorek; Instagram Zostań z Vintage – Krzesło GFM-22 typ 200/128</t>
+  </si>
+  <si>
     <t>nerkowate tapicerowane oparcie; oparcie szersze od wspornika; smukłe zwężające się nogi; lekka ażurowa konstrukcja; gięta drewniana rama; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; cienkie elementy konstrukcyjne; szeroko rozstawione tylne nogi; profil boczny z delikatnie pochylonym oparciem; organiczny kształt oparcia; minimalistyczna sylwetka lat 60.</t>
   </si>
   <si>
+    <t>Typ 1020</t>
+  </si>
+  <si>
+    <t>Muszelka</t>
+  </si>
+  <si>
+    <t>Wiesław Leśniewski; Stanisław Lejkowski</t>
+  </si>
+  <si>
+    <t>Słupskie Fabryki Mebli</t>
+  </si>
+  <si>
+    <t>muszelkowe profilowane oparcie; jednolita tapicerowana skorupa; zaokrąglona górna krawędź oparcia; smukłe stożkowe nogi; lekka modernistyczna forma; brak podłokietników; organiczna sylwetka</t>
+  </si>
+  <si>
+    <t>profilowana skorupa ze sklejki; tapicerowana skorupa; drewniany stelaż; cztery drewniane nogi; konstrukcja szkieletowa; połączenie sklejki i drewna litego</t>
+  </si>
+  <si>
+    <t>RM58; krzesła muszelkowe produkcji NRD; krzesła skandynawskie lat 60.; fotel Ewa</t>
+  </si>
+  <si>
+    <t>krzesła muszelkowe Słupskich Fabryk Mebli; projekty Wiesława Leśniewskiego i Stanisława Lejkowskiego; meble ze sklejki profilowanej produkowane przez SFM</t>
+  </si>
+  <si>
+    <t>Archiwalne katalogi Słupskich Fabryk Mebli; opracowania kolekcjonerskie dotyczące wzornictwa SFM; materiały renowatorów specjalizujących się w meblach PRL; publikacje poświęcone projektom Wiesława Leśniewskiego i Stanisława Lejkowskiego</t>
+  </si>
+  <si>
     <t>muszelkowe profilowane oparcie; jednolita tapicerowana skorupa; zaokrąglona górna krawędź oparcia; płynne przejście oparcia w siedzisko; brak podłokietników; cztery smukłe stożkowe drewniane nogi; lekka organiczna bryła; profilowana skorupa ze sklejki; niewielki prześwit pod siedziskiem; forma inspirowana muszlą</t>
   </si>
   <si>
+    <t>Bumerang</t>
+  </si>
+  <si>
+    <t>Ryszard Kulm</t>
+  </si>
+  <si>
+    <t>przełom lat 50. i 60. XX w.; produkcja seryjna od początku lat 60</t>
+  </si>
+  <si>
+    <t>Gościcińska Fabryka Mebli</t>
+  </si>
+  <si>
+    <t>charakterystyczne łukowato wygięte przednie nogi przypominające bumerang; lekka ażurowa konstrukcja; tapicerowane siedzisko; tapicerowane oparcie; smukła sylwetka; zwężające się ku dołowi nogi; modernistyczna forma inspirowana skandynawskim wzornictwem</t>
+  </si>
+  <si>
+    <t>drewniany stelaż bukowy; gięte elementy boczne; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; połączenia skręcane i klejone</t>
+  </si>
+  <si>
+    <t>GFM-22; typ 200-190 Rajmunda Hałasa; GFM-57 Skoczek; krzesła skandynawskie lat 60</t>
+  </si>
+  <si>
+    <t>krzesła Gościcińskiej Fabryki Mebli; wariant 299XB (Do weryfikacji); rodzina krzeseł Bumerang</t>
+  </si>
+  <si>
+    <t>Meblostan – Komplet 4 krzeseł Bumerang typ 299; Skarby PRL – Krzesło tapicerowane Bumerang typ 299; Patyna – Komplet krzeseł typ 299 Bumerang; Deccoria – 10 słynnych mebli z PRL; Stary Fotel – Krzesła Bumerang metamorfoza</t>
+  </si>
+  <si>
     <t>łukowato wygięte przednie nogi w kształcie bumerangu; gięte boczne elementy drewniane; tapicerowane prostokątne siedzisko; tapicerowane oparcie; smukła lekka bryła; cienki drewniany stelaż; zwężające się ku dołowi nogi; wyraźny prześwit pod siedziskiem; organiczny profil boczny; lekko odchylone oparcie; minimalistyczna forma lat 60.; charakterystyczna sylwetka bumerangu</t>
   </si>
   <si>
+    <t>Typ 300-227</t>
+  </si>
+  <si>
+    <t>Celia</t>
+  </si>
+  <si>
+    <t>ok. 1965; produkcja na przełomie lat 60. i 70. XX w.</t>
+  </si>
+  <si>
+    <t>Zamojskie Fabryki Mebli</t>
+  </si>
+  <si>
+    <t>brak podłokietników; toczone drewniane nogi umieszczone po bokach części tapicerowanej; trapezowe siedzisko; proste tapicerowane oparcie; lekka minimalistyczna forma; kompaktowe wymiary; stylistyka skandynawskiego modernizmu</t>
+  </si>
+  <si>
+    <t>drewniany stelaż; toczone nogi; tapicerowane siedzisko; tapicerowane oparcie; otwarta konstrukcja bez podłokietników; konstrukcja szkieletowa przeznaczona do produkcji seryjnej</t>
+  </si>
+  <si>
+    <t>typ 300-190 Lisek; typ 366; GFM-64; lekkie fotele klubowe PRL bez podłokietników</t>
+  </si>
+  <si>
+    <t>fotele Zamojskich Fabryk Mebli z lat 60. i 70.; meble klubowe produkowane w Zamościu; modele o minimalistycznej konstrukcji bez podłokietników</t>
+  </si>
+  <si>
+    <t>Meblostan – Fotel CELIA typ 300-227; Patyna – Fotel CELIA typ 300-227 PRL; Szajba Sklep – Fotel Celia typ 300-227; materiały kolekcjonerskie dotyczące Zamojskich Fabryk Mebli</t>
+  </si>
+  <si>
     <t>brak podłokietników; toczone drewniane nogi umieszczone po bokach korpusu; trapezowe tapicerowane siedzisko; prostokątne tapicerowane oparcie; lekka minimalistyczna bryła; duży prześwit pod siedziskiem; cienki drewniany stelaż; zwężające się ku dołowi nogi; odsłonięte drewniane elementy boczne; kompaktowe proporcje; geometryczny profil boczny; forma inspirowana skandynawskim modernizmem</t>
   </si>
   <si>
+    <t>Typ 300-139</t>
+  </si>
+  <si>
+    <t>Stefan</t>
+  </si>
+  <si>
+    <t>Swarzędzka Fabryka Mebli</t>
+  </si>
+  <si>
+    <t>szerokie drewniane podłokietniki o łagodnym łuku; otwarta konstrukcja boczna; luźne tapicerowane poduchy siedziska i oparcia; rozłożysta bryła; lekka skandynawska stylistyka; nisko osadzone siedzisko; masywny drewniany stelaż</t>
+  </si>
+  <si>
+    <t>stelaż z litego drewna bukowego; otwarta rama boczna; osobna poduszka siedziska; osobna poduszka oparcia; pasy tapicerskie; konstrukcja szkieletowa skręcana</t>
+  </si>
+  <si>
+    <t>typ 300-123 Puchała; typ 366; duńskie fotele Kandidaten projektu Ib Kofod-Larsena; fotele skandynawskie lat 60</t>
+  </si>
+  <si>
+    <t>sofa Stefan; zestawy wypoczynkowe Swarzędzkiej Fabryki Mebli; meble eksportowe Swarzędzkiej Fabryki Mebli z lat 60.</t>
+  </si>
+  <si>
+    <t>„Meble w produkcji 1962” – Zjednoczenie Przemysłu Meblarskiego; „Meble do małych mieszkań. Informator”, Wydawnictwo Katalogów i Cenników 1966; Laminerva – „Ikony polskiego designu: Fotel Stefan typ 300-139”; Meblostan – Para foteli Stefan typ 300-139; Patyna – Para foteli Stefan typ 300-139</t>
+  </si>
+  <si>
     <t>szerokie wyprofilowane drewniane podłokietniki; otwarta drewniana rama boczna; luźna poduszka siedziska; luźna poduszka oparcia; nisko osadzone głębokie siedzisko; prostokątne grube poduchy; lekko odchylone oparcie; masywny bukowy stelaż; duży prześwit pod siedziskiem; szeroki rozstaw przednich nóg; profil boczny inspirowany wzornictwem skandynawskim; rozłożysta bryła eksportowa</t>
   </si>
   <si>
+    <t>B-3300</t>
+  </si>
+  <si>
+    <t>ok. 1969; produkcja w końcu lat 60. i na początku lat 70. XX w</t>
+  </si>
+  <si>
+    <t>Zakład Mebli Giętych w Radomsku; Fabryki Mebli Radomsko (późniejsze nazewnictwo zakładu)</t>
+  </si>
+  <si>
+    <t>gięte drewniane podłokietniki; szerokie tapicerowane siedzisko; prostokątne tapicerowane oparcie; otwarta konstrukcja boczna; gięty bukowy stelaż; nisko osadzona bryła; elegancka modernistyczna forma</t>
+  </si>
+  <si>
+    <t>stelaż z giętego drewna bukowego; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; elementy gięte wykonane w technologii Thoneta; konstrukcja skręcana</t>
+  </si>
+  <si>
+    <t>B-310 VAR; B-6028; GFM-64; typ 300-139 Stefan</t>
+  </si>
+  <si>
+    <t>fotele Zakładu Mebli Giętych w Radomsku; modele eksportowe Radomsko z lat 60. i 70.; rodzina foteli z giętego drewna bukowego</t>
+  </si>
+  <si>
+    <t>Patyna – Fotel B-3300 Zakład Mebli Giętych w Radomsku; Meblostan – Para foteli B-3300; archiwalne materiały Fabryk Mebli Radomsko; oferty kolekcjonerskie dokumentujące oryginalne oznaczenie modelu</t>
+  </si>
+  <si>
     <t>gięte drewniane podłokietniki; otwarta drewniana rama boczna; szerokie prostokątne oparcie; szerokie głębokie siedzisko; bukowy gięty stelaż; duży prześwit pod siedziskiem; łagodnie wygięte boki; zwężające się ku dołowi nogi; lekko pochylone oparcie; masywniejsza bryła niż typ 366; widoczne elementy z giętego drewna; modernistyczna forma gabinetowa</t>
+  </si>
+  <si>
+    <t>Cechy AI</t>
   </si>
 </sst>
 </file>
@@ -1031,9 +1028,48 @@
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="20">
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1346,7 +1382,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAC340A0-F689-4CF5-934F-277213A09CD2}" name="Tabela1" displayName="Tabela1" ref="A2:M42" totalsRowShown="0" headerRowDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAC340A0-F689-4CF5-934F-277213A09CD2}" name="Tabela1" displayName="Tabela1" ref="A2:M42" totalsRowShown="0" headerRowDxfId="19">
   <autoFilter ref="A2:M42" xr:uid="{AAC340A0-F689-4CF5-934F-277213A09CD2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:M8">
     <sortCondition ref="C2:C8"/>
@@ -1360,7 +1396,7 @@
     <tableColumn id="5" xr3:uid="{FC87805C-8F21-4877-A2BB-F94A46848488}" name="Top3 contains"/>
     <tableColumn id="12" xr3:uid="{083260FC-C283-425D-8992-A120FCD63F58}" name="Model Family"/>
     <tableColumn id="6" xr3:uid="{C375EF1E-B099-4419-8B9C-B2440FD0A8ED}" name="Designer"/>
-    <tableColumn id="7" xr3:uid="{DD17F6C6-7610-4EE0-A977-F8A13F1B8EBA}" name="Confidence" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{DD17F6C6-7610-4EE0-A977-F8A13F1B8EBA}" name="Confidence" dataDxfId="18"/>
     <tableColumn id="8" xr3:uid="{B609250C-19DF-4BCE-8148-69FA85A5C4D5}" name="Error Type"/>
     <tableColumn id="9" xr3:uid="{7ECB45DF-B162-4E08-85FE-5889D14F4EA2}" name="Notes"/>
     <tableColumn id="10" xr3:uid="{7DB3FB91-9C91-4420-A0AD-58F455F6AD18}" name="Severity"/>
@@ -1371,22 +1407,23 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0B9BF425-AAE6-496E-A318-81223EDA70A0}" name="Table2" displayName="Table2" ref="A1:M21" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
-  <autoFilter ref="A1:M21" xr:uid="{0B9BF425-AAE6-496E-A318-81223EDA70A0}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{BEC8128C-B6F8-41AF-8B4E-AC51172C6F9B}" name="ID" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{A4D5EBAD-8137-4068-9AB3-4017AE021691}" name="Model" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{2E31A0DA-DF43-4372-8896-81E05381952A}" name="Potoczna nazwa" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{BFBF567B-85D5-410F-86B7-E7A5AE9C3740}" name="Projektant" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{C0BA823A-68AD-4568-86DC-D7A0821FE81E}" name="Rok" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{A85EDE16-4C80-416A-961D-E6418592861C}" name="Typ" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{B6F3255D-9933-44DB-84CE-345F6ADC20CF}" name="Producent" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{444D790F-7610-4FF6-B3B8-84C2F85CD109}" name="Cechy Charakterystyczne" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{98CF13B3-BB3C-451C-BD71-AA322E9D297B}" name="Konstrukcja" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{CED6A324-3FA7-4066-97E4-A5BE6D00D638}" name="Mylony z" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{7D23AC8B-5C76-4D9D-94A1-5E0E701AC60B}" name="Rodzina modeli" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{6E7FC306-D5DA-4E3A-8481-0DE3695A5890}" name="Źródła" dataDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{86F52982-86F4-44FD-8A46-84423C74DFF2}" name="Poziom pewności" dataDxfId="1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0B9BF425-AAE6-496E-A318-81223EDA70A0}" name="Table2" displayName="Table2" ref="A1:N21" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+  <autoFilter ref="A1:N21" xr:uid="{0B9BF425-AAE6-496E-A318-81223EDA70A0}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{BEC8128C-B6F8-41AF-8B4E-AC51172C6F9B}" name="ID" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{A4D5EBAD-8137-4068-9AB3-4017AE021691}" name="Model" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{2E31A0DA-DF43-4372-8896-81E05381952A}" name="Potoczna nazwa" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{BFBF567B-85D5-410F-86B7-E7A5AE9C3740}" name="Projektant" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{C0BA823A-68AD-4568-86DC-D7A0821FE81E}" name="Rok" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{A85EDE16-4C80-416A-961D-E6418592861C}" name="Typ" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{B6F3255D-9933-44DB-84CE-345F6ADC20CF}" name="Producent" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{444D790F-7610-4FF6-B3B8-84C2F85CD109}" name="Cechy Charakterystyczne" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{98CF13B3-BB3C-451C-BD71-AA322E9D297B}" name="Konstrukcja" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{CED6A324-3FA7-4066-97E4-A5BE6D00D638}" name="Mylony z" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{7D23AC8B-5C76-4D9D-94A1-5E0E701AC60B}" name="Rodzina modeli" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{6E7FC306-D5DA-4E3A-8481-0DE3695A5890}" name="Źródła" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{86F52982-86F4-44FD-8A46-84423C74DFF2}" name="Poziom pewności" dataDxfId="3"/>
+    <tableColumn id="14" xr3:uid="{633CC391-CD9D-4406-9436-B55C83554066}" name="Search Features" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1396,7 +1433,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{61559DFE-BFDA-476F-A468-7B9F99C28CB5}" name="Table3" displayName="Table3" ref="A1:B21" totalsRowShown="0">
   <autoFilter ref="A1:B21" xr:uid="{61559DFE-BFDA-476F-A468-7B9F99C28CB5}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{27F92EA0-9427-4162-90E8-85D5CAEC32F6}" name="Model"/>
+    <tableColumn id="1" xr3:uid="{27F92EA0-9427-4162-90E8-85D5CAEC32F6}" name="Model" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{67610278-00DF-4DEA-BF65-7097C76D8F9A}" name="Cechy AI" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3080,7 +3117,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E570A043-1276-4CEE-AF12-19208D26EAA5}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -3095,9 +3132,10 @@
     <col min="11" max="11" width="31" customWidth="1"/>
     <col min="12" max="12" width="24.140625" customWidth="1"/>
     <col min="13" max="13" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="5" t="s">
         <v>77</v>
       </c>
@@ -3137,90 +3175,99 @@
       <c r="M1" s="10" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" ht="152.25">
+      <c r="N1" s="10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="409.6">
       <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M2" s="11">
         <v>0.98</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" ht="152.25">
+      <c r="N2" s="9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="409.6">
       <c r="A3" s="9">
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E3" s="9">
         <v>1967</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="M3" s="11">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" ht="152.25">
+      <c r="N3" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="381.75">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -3228,81 +3275,87 @@
         <v>26</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="M4" s="11">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" ht="213">
+      <c r="N4" s="9" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="409.6">
       <c r="A5" s="9">
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="M5" s="11">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" ht="106.5">
+      <c r="N5" s="9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="321">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -3310,366 +3363,393 @@
         <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E6" s="9">
         <v>1962</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="M6" s="11">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" ht="152.25">
+      <c r="N6" s="9" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="409.6">
       <c r="A7" s="9">
         <v>6</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="M7" s="11">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" ht="137.25">
+      <c r="N7" s="9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="409.6">
       <c r="A8" s="9">
         <v>7</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E8" s="9">
         <v>1958</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="M8" s="11">
         <v>0.99</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" ht="91.5">
+      <c r="N8" s="9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="366">
       <c r="A9" s="9">
         <v>8</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="M9" s="11">
         <v>0.92</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" ht="137.25">
+      <c r="N9" s="9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="409.6">
       <c r="A10" s="9">
         <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="M10" s="11">
         <v>0.87</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" ht="137.25">
+      <c r="N10" s="9" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="409.6">
       <c r="A11" s="9">
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="E11" s="9">
         <v>1965</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="M11" s="11">
         <v>0.96</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" ht="152.25">
+      <c r="N11" s="9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="409.6">
       <c r="A12" s="9">
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="M12" s="11">
         <v>0.94</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" ht="183">
+      <c r="N12" s="9" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="409.6">
       <c r="A13" s="9">
         <v>12</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="M13" s="11">
         <v>0.96</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" ht="229.5">
+      <c r="N13" s="9" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="366">
       <c r="A14" s="9">
         <v>13</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="9" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="M14" s="11">
         <v>0.72</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" ht="137.25">
+      <c r="N14" s="9" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="409.6">
       <c r="A15" s="9">
         <v>14</v>
       </c>
@@ -3678,117 +3758,126 @@
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="M15" s="11">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" ht="137.25">
+      <c r="N15" s="9" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="396.75">
       <c r="A16" s="9">
         <v>15</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="M16" s="11">
         <v>0.93</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" ht="167.25">
+      <c r="N16" s="9" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="321">
       <c r="A17" s="9">
         <v>16</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>228</v>
+        <v>244</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="E17" s="9">
         <v>1962</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>231</v>
+        <v>247</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>234</v>
+        <v>250</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>235</v>
+        <v>251</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="M17" s="11">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" ht="152.25">
+      <c r="N17" s="9" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="381.75">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -3796,152 +3885,164 @@
         <v>67</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>237</v>
+        <v>254</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>238</v>
+        <v>255</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>239</v>
+        <v>256</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>240</v>
+        <v>257</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>241</v>
+        <v>258</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>242</v>
+        <v>259</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>243</v>
+        <v>260</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>244</v>
+        <v>261</v>
       </c>
       <c r="L18" s="9" t="s">
-        <v>245</v>
+        <v>262</v>
       </c>
       <c r="M18" s="11">
         <v>0.91</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" ht="121.5">
+      <c r="N18" s="9" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="409.6">
       <c r="A19" s="9">
         <v>18</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="C19" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>249</v>
+        <v>267</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>250</v>
+        <v>268</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>252</v>
+        <v>270</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
       <c r="M19" s="11">
         <v>0.95</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" ht="213">
+      <c r="N19" s="9" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="396.75">
       <c r="A20" s="9">
         <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>255</v>
+        <v>274</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>256</v>
+        <v>275</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>257</v>
+        <v>276</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>258</v>
+        <v>277</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>259</v>
+        <v>278</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>260</v>
+        <v>279</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>262</v>
+        <v>281</v>
       </c>
       <c r="M20" s="11">
         <v>0.95</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" ht="137.25">
+      <c r="N20" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="366">
       <c r="A21" s="9">
         <v>20</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>263</v>
+        <v>283</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9" t="s">
-        <v>264</v>
+        <v>284</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>265</v>
+        <v>285</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>266</v>
+        <v>286</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>267</v>
+        <v>287</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>268</v>
+        <v>288</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>270</v>
+        <v>290</v>
       </c>
       <c r="M21" s="11">
         <v>0.86</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -3966,167 +4067,167 @@
         <v>78</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>271</v>
+        <v>292</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="106.5">
-      <c r="A2">
-        <v>366</v>
+      <c r="A2" s="9" t="s">
+        <v>91</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>272</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="91.5">
-      <c r="A3" t="s">
+      <c r="A3" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="91.5">
+      <c r="A4" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="91.5">
+      <c r="A5" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="76.5">
+      <c r="A6" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="91.5">
+      <c r="A7" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="106.5">
+      <c r="A8" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="76.5">
+      <c r="A9" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="152.25">
+      <c r="A10" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="183">
+      <c r="A11" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="91.5">
+      <c r="A12" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="91.5">
+      <c r="A13" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="76.5">
+      <c r="A14" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="91.5">
+      <c r="A15" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="91.5">
+      <c r="A16" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="76.5">
+      <c r="A17" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="91.5">
+      <c r="A18" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="91.5">
+      <c r="A19" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B3" s="1" t="s">
+    </row>
+    <row r="20" spans="1:2" ht="91.5">
+      <c r="A20" s="9" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="91.5">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="91.5">
-      <c r="A5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="76.5">
-      <c r="A6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="91.5">
-      <c r="A7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="106.5">
-      <c r="A8" t="s">
-        <v>146</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="76.5">
-      <c r="A9" t="s">
-        <v>155</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="152.25">
-      <c r="A10" t="s">
-        <v>165</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="183">
-      <c r="A11" t="s">
+      <c r="B20" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="B11" s="1" t="s">
+    </row>
+    <row r="21" spans="1:2" ht="76.5">
+      <c r="A21" s="9" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="91.5">
-      <c r="A12" t="s">
-        <v>184</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="91.5">
-      <c r="A13" t="s">
-        <v>193</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="76.5">
-      <c r="A14" t="s">
-        <v>203</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="91.5">
-      <c r="A15" t="s">
-        <v>60</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="91.5">
-      <c r="A16" t="s">
-        <v>62</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="76.5">
-      <c r="A17" t="s">
-        <v>228</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="91.5">
-      <c r="A18" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="91.5">
-      <c r="A19" t="s">
-        <v>246</v>
-      </c>
-      <c r="B19" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="91.5">
-      <c r="A20" t="s">
-        <v>255</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="76.5">
-      <c r="A21" t="s">
-        <v>263</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add hard filters to candidate search
</commit_message>
<xml_diff>
--- a/data/furniture.xlsx
+++ b/data/furniture.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98AB1377-DA10-4E8D-9E0C-6724EC958207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3147F11-BFBA-4623-B963-325CD87AC8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark" sheetId="1" r:id="rId1"/>
@@ -337,10 +337,10 @@
     <t>Dolnośląska Fabryka Mebli w Świebodzicach</t>
   </si>
   <si>
-    <t>drewniane boczki pełniące funkcję nóg i podłokietników; lekka modernistyczna forma; trapezowe siedzisko; trapezowe oparcie; widoczne elementy drewniane; oddzielne moduły tapicerowane; niewielkie gabaryty</t>
-  </si>
-  <si>
-    <t>drewniana konstrukcja nośna; boczki z litego drewna; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja przeznaczona do produkcji seryjnej</t>
+    <t>Fotel składa się z tapicerowanej „łupiny” tworzonej przez zintegrowane siedzisko i oparcie. Po rozłożeniu jej obrys przypomina trapez o lekko wyokrąglonych bokach i narożnikach. Boczne podpory wykonane z drewna łączą po dwie zwężające się ku dołowi nogi z wyoblonym podłokietnikiem o organicznym kształcie. Mebel pozbawiony jest dekoracyjnych elementów. Tapicerkę zdobią wyłącznie guziki pikowania, natomiast elementy drewniane posiadają widoczne śruby o dużych główkach. Poszczególne egzemplarze różnią się tkaniną obiciową, gatunkiem drewna, kolorem lakieru oraz występują także warianty z czarno malowanymi podłokietnikami.</t>
+  </si>
+  <si>
+    <t>Konstrukcja składa się z tapicerowanej łupiny zintegrowanego siedziska i oparcia oraz dwóch drewnianych podpór bocznych. Każda podpora stanowi element łączący podłokietnik z dwiema nogami. W wersji produkcyjnej zastosowano widoczne połączenia śrubowe zamiast projektowanych niewidocznych mocowań.</t>
   </si>
   <si>
     <t>GFM-64; RM58; polskie fotele klubowe lat 60.</t>
@@ -352,7 +352,31 @@
     <t>opracowania dotyczące Józefa Chierowskiego; dokumentacja 366 Concept; zbiory Muzeum Narodowego w Warszawie; Polski New Look Ewa Solarz i Agnieszka Sural; publikacje o polskim wzornictwie powojennym</t>
   </si>
   <si>
-    <t>drewniane boczki tworzące nogi i podłokietniki; trapezowe oparcie zwężające się ku górze; trapezowe siedzisko zwężające się ku tyłowi; widoczny prześwit pod siedziskiem; oddzielne moduły tapicerowanego siedziska i oparcia; skośnie rozstawione nogi; pozioma linia podłokietników; odsłonięte drewniane elementy boczne; lekka geometryczna bryła; brak tapicerowanych boków; zwężające się ku dołowi nogi; charakterystyczny profil boczny w kształcie odwróconego V</t>
+    <t>drewniane boczki;
+otwarta rama boczna;
+widoczna drewniana rama;
+tapicerowana łupina;
+jednolita łupina;
+zintegrowane siedzisko;
+zintegrowane oparcie;
+trapezowy obrys korpusu;
+zaokrąglone narożniki korpusu;
+zaokrąglone boki korpusu;
+tapicerowane siedzisko;
+tapicerowane oparcie;
+wyoblone podłokietniki;
+organiczny kształt podłokietników;
+drewniane podłokietniki;
+zwężające się nogi;
+skośnie rozstawione nogi;
+cztery drewniane nogi;
+widoczne śruby;
+duże główki śrub;
+guziki pikowania;
+prześwit pod siedziskiem;
+odsłonięta drewniana konstrukcja;
+widoczne drewniane elementy;
+brak ozdobnych detali</t>
   </si>
   <si>
     <t>Fotel typ 300-190</t>
@@ -367,10 +391,10 @@
     <t>Dolnośląska Fabryka Mebli w Świebodzicach; Bystrzyckie Fabryki Mebli; Zakład Mebli Giętych FAMEG Radomsko; Świdnicki Ośrodek Przemysłu Meblarskiego</t>
   </si>
   <si>
-    <t>smukła lekka sylwetka; płaskie drewniane podłokietniki; toczone nogi zwężające się ku dołowi; widoczna drewniana rama boczna; prostokątne tapicerowane oparcie; kompaktowe wymiary; modernistyczna forma</t>
-  </si>
-  <si>
-    <t>konstrukcja nośna z drewna bukowego; toczone nogi mocowane do podłokietników; poprzeczne belki usztywniające ramę; pasy tapicerskie; formatki gumowe jako wypełnienie; lakierowane elementy drewniane</t>
+    <t>Fotel posiada lekką, smukłą konstrukcję opartą na odsłoniętej drewnianej ramie. Tapicerowane siedzisko i oparcie osadzone są pomiędzy drewnianymi boczkami zakończonymi płaskimi podłokietnikami. Konstrukcja wsparta jest na czterech toczonych, lekko zwężających się nogach. W połowie wysokości nóg widoczne są poprzeczne belki tworzące charakterystyczną ramę usztywniającą. Drewniane elementy wykończone były lakierem o wykończeniu matowym, półmatowym lub z połyskiem.</t>
+  </si>
+  <si>
+    <t>Konstrukcję nośną tworzą drewniane boczki połączone poprzecznymi belkami oraz stelażem. Nogi są mocowane do płaskich podłokietników. Do wykonania stolarki zastosowano drewno bukowe. Siedzisko wykorzystuje formatki gumowe osadzone na elastycznych pasach zamiast sprężyn i tradycyjnych wypełnień.</t>
   </si>
   <si>
     <t>typ 366; GFM-64; fotele klubowe PRL z lat 60.</t>
@@ -382,7 +406,31 @@
     <t>Nowohuckie Renowacje – Fotel Lisek typ 300-190; Conchita Home – 4 fotele z PRL które musisz znać; dokumentacja i opisy egzemplarzy Typ 300-190; archiwalne materiały producentów cytowane w opracowaniach specjalistycznych</t>
   </si>
   <si>
-    <t>płaskie drewniane podłokietniki; toczone nogi zwężające się ku dołowi; nogi przechodzące przez podłokietniki; widoczna prostokątna rama boczna; poziome poprzeczki między nogami; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; smukła lekka bryła; odsłonięta konstrukcja drewniana; niskie podłokietniki; geometryczny profil boczny</t>
+    <t>toczone nogi;
+lekko zwężające się nogi;
+cztery drewniane nogi;
+drewniane boczki;
+otwarta rama boczna;
+widoczna drewniana rama;
+poprzeczne belki;
+widoczne belki między nogami;
+płaskie podłokietniki;
+drewniane podłokietniki;
+odsłonięta konstrukcja;
+prześwit pod siedziskiem;
+tapicerowane siedzisko;
+tapicerowane oparcie;
+prostokątne oparcie;
+prostokątne siedzisko;
+smukła bryła;
+wysokie oparcie;
+widoczne boczne podpory;
+drewniany stelaż;
+proste linie konstrukcji;
+otwarte boki;
+rama usztywniająca;
+widoczna konstrukcja pod siedziskiem;
+minimalistyczna forma</t>
   </si>
   <si>
     <t>Do weryfikacji; często błędnie określany jako „Lisek”</t>
@@ -397,10 +445,10 @@
     <t>Zakłady Przemysłu Meblarskiego im. Gwardii Ludowej w Radomsku; Fabryki Mebli Radomsko</t>
   </si>
   <si>
-    <t>otwarta drewniana rama boczna; prostokątne tapicerowane siedzisko; szerokie tapicerowane oparcie; toczone okrągłe nogi; nisko osadzone siedzisko; lekka konstrukcja szkieletowa; widoczne drewniane podłokietniki</t>
-  </si>
-  <si>
-    <t>rama z drewna bukowego; toczone elementy nóg; tapicerowane siedzisko montowane śrubami; tapicerowane oparcie montowane śrubami; wewnętrzny szkielet z drewna iglastego; konstrukcja rozbieralna</t>
+    <t>Fotel posiada otwartą drewnianą konstrukcję zewnętrzną wykonaną z litego drewna. Tapicerowane siedzisko i oparcie zamocowane są wewnątrz drewnianej ramy za pomocą wkrętów lub śrub. Konstrukcja opiera się na czterech toczonych nogach połączonych belkami podtrzymującymi siedzisko. Charakterystycznym elementem są zaokrąglone drewniane podłokietniki stanowiące integralną część bocznej ramy.</t>
+  </si>
+  <si>
+    <t>Konstrukcja wykonana jest z litej tarcicy bukowej. Szkielet ukryty pod tapicerką wykonano z tarcicy iglastej. Siedzisko i oparcie mocowane są do ramy za pomocą wkrętów lub śrub. Połączenia konstrukcyjne obejmują połączenia czopowe oraz połączenia na wkręty. W siedzisku zastosowano pasy tapicerskie i tworzywo piankowe.</t>
   </si>
   <si>
     <t>typ 300-190 Lisek; BW-14; typ 366</t>
@@ -412,7 +460,30 @@
     <t>Patyna.pl – fotel B-7727 Radomsko PRL; Meblostan – fotel B-7727; Nowohuckie Renowacje – fotel B-7727; Vilandy – fotel Lis typ B-7727; Allegro – fotel PRL model B-7727 Radomsko lata 70; Reko-Czyny – identyfikacja fotela B-7727</t>
   </si>
   <si>
-    <t>otwarta drewniana rama boczna; prostokątne szerokie oparcie; oparcie szersze niż w modelu 300-190; prostokątne siedzisko; okrągłe toczone nogi; poziome drewniane podłokietniki; widoczne połączenia ramy bocznej; duży prześwit pod siedziskiem; lekka geometryczna bryła; drewniane belki łączące nogi; rozbieralne moduły siedziska i oparcia; nisko osadzone siedzisko</t>
+    <t>toczone nogi;
+cztery drewniane nogi;
+zaokrąglone podłokietniki;
+drewniane podłokietniki;
+otwarta rama boczna;
+widoczna drewniana rama;
+drewniane boczki;
+belki pod siedziskiem;
+widoczne belki;
+tapicerowane siedzisko;
+tapicerowane oparcie;
+oddzielne siedzisko;
+oddzielne oparcie;
+prostokątne oparcie;
+prostokątne siedzisko;
+widoczne śruby;
+widoczne wkręty;
+prześwit pod siedziskiem;
+odsłonięta drewniana konstrukcja;
+rama zewnętrzna;
+otwarte boki;
+widoczne mocowanie siedziska;
+widoczne mocowanie oparcia;
+drewniany stelaż</t>
   </si>
   <si>
     <t>Typ 300-177</t>
@@ -457,10 +528,10 @@
     <t>Strzeleckie Zakłady Przemysłu Terenowego w Strzelcach Opolskich</t>
   </si>
   <si>
-    <t>stalowy stelaż; muszelkowa forma korpusu; kubełkowe siedzisko; smukłe wykręcane nogi; ruchome stopki kulowe; lekka wizualnie konstrukcja; obłe linie oparcia</t>
-  </si>
-  <si>
-    <t>spawana rama z prętów stalowych; tapicerowany korpus; cztery stalowe wykręcane nogi; siedzisko na pasach tapicerskich; konstrukcja metalowa bez drewnianych boczków</t>
+    <t>Fotel posiada muszelkowy, kubełkowy korpus tworzący jednolitą tapicerowaną bryłę. Szerokie, półkoliste oparcie płynnie przechodzi w siedzisko, nadając bryle profil przypominający muszlę. Korpus osadzony jest na odsłoniętym stalowym stelażu wspartym na czterech smukłych metalowych nogach. Fotel nie posiada drewnianych podłokietników, a wysoka podstawa nadaje konstrukcji lekką formę.</t>
+  </si>
+  <si>
+    <t>Konstrukcję nośną stanowi rama wykonana ze spawanych prętów stalowych. Rama wsparta jest na czterech stalowych, wykręcanych nogach zakończonych ruchomymi stopkami. W modelu Koeln 1 zastosowano pojedynczą stalową nogę obrotową.</t>
   </si>
   <si>
     <t>fotel Köln 1; fotel Muszelka; fotele klubowe na stelażu stalowym z lat 60.</t>
@@ -472,7 +543,31 @@
     <t>Meblostan – Para foteli tapicerowanych EWA; Odnowa Mebli – Fotel Ewa; Patyna.pl – Komplet foteli typ Ewa; materiały kolekcjonerskie rynku vintage</t>
   </si>
   <si>
-    <t>muszelkowy korpus; kubełkowe siedzisko; zaokrąglone oparcie; stalowy stelaż; cztery smukłe metalowe nogi; wykręcane nogi; kulowe stopki; brak drewnianych podłokietników; jednolita tapicerowana bryła; szerokie półkoliste oparcie; lekka forma na wysokich nogach; profil przypominający muszlę</t>
+    <t>muszelkowy korpus;
+kubełkowe siedzisko;
+jednolita tapicerowana bryła;
+tapicerowane siedzisko;
+tapicerowane oparcie;
+zaokrąglone oparcie;
+szerokie półkoliste oparcie;
+profil przypominający muszlę;
+stalowy stelaż;
+stalowa rama;
+rama z prętów stalowych;
+spawana rama;
+odsłonięty stalowy stelaż;
+widoczna stalowa konstrukcja;
+cztery metalowe nogi;
+smukłe metalowe nogi;
+wysokie nogi;
+wykręcane nogi;
+kulowe stopki;
+ruchome stopki;
+prześwit pod siedziskiem;
+brak drewnianych podłokietników;
+otwarta konstrukcja;
+obszerne siedzisko;
+obszerne oparcie</t>
   </si>
   <si>
     <t>Typ 300-123</t>
@@ -1026,7 +1121,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="20">
     <dxf>
@@ -3267,7 +3362,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="381.75">
+    <row r="4" spans="1:14" ht="409.6">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -3355,7 +3450,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="321">
+    <row r="6" spans="1:14" ht="409.6">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -4070,7 +4165,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="106.5">
+    <row r="2" spans="1:2" ht="381.75">
       <c r="A2" s="9" t="s">
         <v>91</v>
       </c>
@@ -4078,7 +4173,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="91.5">
+    <row r="3" spans="1:2" ht="381.75">
       <c r="A3" s="9" t="s">
         <v>103</v>
       </c>
@@ -4086,7 +4181,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="91.5">
+    <row r="4" spans="1:2" ht="366">
       <c r="A4" s="9" t="s">
         <v>26</v>
       </c>
@@ -4102,7 +4197,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="76.5">
+    <row r="6" spans="1:2" ht="381.75">
       <c r="A6" s="9" t="s">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
feat: add reference-image verification stage to identification pipeline
</commit_message>
<xml_diff>
--- a/data/furniture.xlsx
+++ b/data/furniture.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3147F11-BFBA-4623-B963-325CD87AC8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B691E158-FE89-466B-8953-B0ED820191F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="294">
   <si>
     <t>Prompt 1</t>
   </si>
@@ -284,6 +284,9 @@
   </si>
   <si>
     <t>Potoczna nazwa</t>
+  </si>
+  <si>
+    <t>REFERENCE_ID</t>
   </si>
   <si>
     <t>Projektant</t>
@@ -1123,7 +1126,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="21">
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1164,6 +1167,25 @@
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1477,7 +1499,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAC340A0-F689-4CF5-934F-277213A09CD2}" name="Tabela1" displayName="Tabela1" ref="A2:M42" totalsRowShown="0" headerRowDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAC340A0-F689-4CF5-934F-277213A09CD2}" name="Tabela1" displayName="Tabela1" ref="A2:M42" totalsRowShown="0" headerRowDxfId="20">
   <autoFilter ref="A2:M42" xr:uid="{AAC340A0-F689-4CF5-934F-277213A09CD2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:M8">
     <sortCondition ref="C2:C8"/>
@@ -1491,7 +1513,7 @@
     <tableColumn id="5" xr3:uid="{FC87805C-8F21-4877-A2BB-F94A46848488}" name="Top3 contains"/>
     <tableColumn id="12" xr3:uid="{083260FC-C283-425D-8992-A120FCD63F58}" name="Model Family"/>
     <tableColumn id="6" xr3:uid="{C375EF1E-B099-4419-8B9C-B2440FD0A8ED}" name="Designer"/>
-    <tableColumn id="7" xr3:uid="{DD17F6C6-7610-4EE0-A977-F8A13F1B8EBA}" name="Confidence" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{DD17F6C6-7610-4EE0-A977-F8A13F1B8EBA}" name="Confidence" dataDxfId="19"/>
     <tableColumn id="8" xr3:uid="{B609250C-19DF-4BCE-8148-69FA85A5C4D5}" name="Error Type"/>
     <tableColumn id="9" xr3:uid="{7ECB45DF-B162-4E08-85FE-5889D14F4EA2}" name="Notes"/>
     <tableColumn id="10" xr3:uid="{7DB3FB91-9C91-4420-A0AD-58F455F6AD18}" name="Severity"/>
@@ -1502,12 +1524,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0B9BF425-AAE6-496E-A318-81223EDA70A0}" name="Table2" displayName="Table2" ref="A1:N21" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
-  <autoFilter ref="A1:N21" xr:uid="{0B9BF425-AAE6-496E-A318-81223EDA70A0}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{BEC8128C-B6F8-41AF-8B4E-AC51172C6F9B}" name="ID" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{A4D5EBAD-8137-4068-9AB3-4017AE021691}" name="Model" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{2E31A0DA-DF43-4372-8896-81E05381952A}" name="Potoczna nazwa" dataDxfId="13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0B9BF425-AAE6-496E-A318-81223EDA70A0}" name="Table2" displayName="Table2" ref="A1:O21" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+  <autoFilter ref="A1:O21" xr:uid="{0B9BF425-AAE6-496E-A318-81223EDA70A0}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{BEC8128C-B6F8-41AF-8B4E-AC51172C6F9B}" name="ID" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{A4D5EBAD-8137-4068-9AB3-4017AE021691}" name="Model" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{2E31A0DA-DF43-4372-8896-81E05381952A}" name="Potoczna nazwa" dataDxfId="14"/>
+    <tableColumn id="16" xr3:uid="{21289632-27BD-4A17-A0EC-06689B74EAF5}" name="REFERENCE_ID" dataDxfId="13"/>
     <tableColumn id="4" xr3:uid="{BFBF567B-85D5-410F-86B7-E7A5AE9C3740}" name="Projektant" dataDxfId="12"/>
     <tableColumn id="5" xr3:uid="{C0BA823A-68AD-4568-86DC-D7A0821FE81E}" name="Rok" dataDxfId="11"/>
     <tableColumn id="6" xr3:uid="{A85EDE16-4C80-416A-961D-E6418592861C}" name="Typ" dataDxfId="10"/>
@@ -3212,25 +3235,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E570A043-1276-4CEE-AF12-19208D26EAA5}">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.5703125" customWidth="1"/>
-    <col min="8" max="8" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.7109375" customWidth="1"/>
-    <col min="10" max="10" width="27" customWidth="1"/>
-    <col min="11" max="11" width="31" customWidth="1"/>
-    <col min="12" max="12" width="24.140625" customWidth="1"/>
-    <col min="13" max="13" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="7" max="7" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.5703125" customWidth="1"/>
+    <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.7109375" customWidth="1"/>
+    <col min="11" max="11" width="27" customWidth="1"/>
+    <col min="12" max="12" width="31" customWidth="1"/>
+    <col min="13" max="13" width="24.140625" customWidth="1"/>
+    <col min="14" max="14" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" s="5" t="s">
         <v>77</v>
       </c>
@@ -3264,7 +3288,7 @@
       <c r="K1" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="L1" s="5" t="s">
         <v>88</v>
       </c>
       <c r="M1" s="10" t="s">
@@ -3273,19 +3297,22 @@
       <c r="N1" s="10" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="409.6">
+      <c r="O1" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="409.6">
       <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D2" s="9" t="s">
         <v>93</v>
+      </c>
+      <c r="D2" s="9">
+        <v>366</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>94</v>
@@ -3311,34 +3338,37 @@
       <c r="L2" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="M2" s="11">
+      <c r="M2" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="N2" s="11">
         <v>0.98</v>
       </c>
-      <c r="N2" s="9" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="409.6">
+      <c r="O2" s="9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="409.6">
       <c r="A3" s="9">
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="D3" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="E3" s="9">
+      <c r="D3" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="F3" s="9">
         <v>1967</v>
       </c>
-      <c r="F3" s="9" t="s">
-        <v>95</v>
-      </c>
       <c r="G3" s="9" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="H3" s="9" t="s">
         <v>107</v>
@@ -3355,14 +3385,17 @@
       <c r="L3" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="M3" s="11">
+      <c r="M3" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="N3" s="11">
         <v>0.88</v>
       </c>
-      <c r="N3" s="9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="409.6">
+      <c r="O3" s="9" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="409.6">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -3370,19 +3403,19 @@
         <v>26</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="D4" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="D4" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>115</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>117</v>
@@ -3399,34 +3432,37 @@
       <c r="L4" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="M4" s="11">
+      <c r="M4" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="N4" s="11">
         <v>0.8</v>
       </c>
-      <c r="N4" s="9" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="409.6">
+      <c r="O4" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="409.6">
       <c r="A5" s="9">
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>126</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>95</v>
+        <v>127</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>127</v>
+        <v>96</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>128</v>
@@ -3443,14 +3479,17 @@
       <c r="L5" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="M5" s="11">
+      <c r="M5" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="N5" s="11">
         <v>0.82</v>
       </c>
-      <c r="N5" s="9" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" ht="409.6">
+      <c r="O5" s="9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="409.6">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -3458,19 +3497,19 @@
         <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="E6" s="9">
+        <v>38</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="F6" s="9">
         <v>1962</v>
       </c>
-      <c r="F6" s="9" t="s">
-        <v>95</v>
-      </c>
       <c r="G6" s="9" t="s">
-        <v>136</v>
+        <v>96</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>137</v>
@@ -3487,37 +3526,40 @@
       <c r="L6" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="M6" s="11">
+      <c r="M6" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="N6" s="11">
         <v>0.85</v>
       </c>
-      <c r="N6" s="9" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" ht="409.6">
+      <c r="O6" s="9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="409.6">
       <c r="A7" s="9">
         <v>6</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>145</v>
+        <v>42</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>146</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>95</v>
+        <v>147</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>148</v>
@@ -3531,34 +3573,37 @@
       <c r="L7" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="M7" s="11">
+      <c r="M7" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="N7" s="11">
         <v>0.9</v>
       </c>
-      <c r="N7" s="9" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="409.6">
+      <c r="O7" s="9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="409.6">
       <c r="A8" s="9">
         <v>7</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="E8" s="9">
+        <v>45</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="F8" s="9">
         <v>1958</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>95</v>
-      </c>
       <c r="G8" s="9" t="s">
-        <v>156</v>
+        <v>96</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>157</v>
@@ -3575,34 +3620,35 @@
       <c r="L8" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="M8" s="11">
+      <c r="M8" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="N8" s="11">
         <v>0.99</v>
       </c>
-      <c r="N8" s="9" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="366">
+      <c r="O8" s="9" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="366">
       <c r="A9" s="9">
         <v>8</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="D9" s="9" t="s">
         <v>165</v>
       </c>
+      <c r="D9" s="9"/>
       <c r="E9" s="9" t="s">
         <v>166</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>95</v>
+        <v>167</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>167</v>
+        <v>96</v>
       </c>
       <c r="H9" s="9" t="s">
         <v>168</v>
@@ -3619,34 +3665,35 @@
       <c r="L9" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="M9" s="11">
+      <c r="M9" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="N9" s="11">
         <v>0.92</v>
       </c>
-      <c r="N9" s="9" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="409.6">
+      <c r="O9" s="9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="409.6">
       <c r="A10" s="9">
         <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>135</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="D10" s="9"/>
       <c r="E10" s="9" t="s">
-        <v>176</v>
+        <v>136</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>95</v>
+        <v>177</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>177</v>
+        <v>96</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>178</v>
@@ -3663,31 +3710,32 @@
       <c r="L10" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="M10" s="11">
+      <c r="M10" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="N10" s="11">
         <v>0.87</v>
       </c>
-      <c r="N10" s="9" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="409.6">
+      <c r="O10" s="9" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="409.6">
       <c r="A11" s="9">
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="D11" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="E11" s="9">
+      <c r="D11" s="9"/>
+      <c r="E11" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="F11" s="9">
         <v>1965</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>187</v>
       </c>
       <c r="G11" s="9" t="s">
         <v>188</v>
@@ -3707,34 +3755,35 @@
       <c r="L11" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="M11" s="11">
+      <c r="M11" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="N11" s="11">
         <v>0.96</v>
       </c>
-      <c r="N11" s="9" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="409.6">
+      <c r="O11" s="9" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="409.6">
       <c r="A12" s="9">
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>93</v>
-      </c>
+        <v>197</v>
+      </c>
+      <c r="D12" s="9"/>
       <c r="E12" s="9" t="s">
-        <v>197</v>
+        <v>94</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>199</v>
@@ -3751,34 +3800,35 @@
       <c r="L12" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="M12" s="11">
+      <c r="M12" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="N12" s="11">
         <v>0.94</v>
       </c>
-      <c r="N12" s="9" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="409.6">
+      <c r="O12" s="9" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="409.6">
       <c r="A13" s="9">
         <v>12</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>206</v>
-      </c>
-      <c r="D13" s="9" t="s">
         <v>207</v>
       </c>
+      <c r="D13" s="9"/>
       <c r="E13" s="9" t="s">
         <v>208</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>187</v>
+        <v>209</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>209</v>
+        <v>188</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>210</v>
@@ -3795,32 +3845,33 @@
       <c r="L13" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="M13" s="11">
+      <c r="M13" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="N13" s="11">
         <v>0.96</v>
       </c>
-      <c r="N13" s="9" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="366">
+      <c r="O13" s="9" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="366">
       <c r="A14" s="9">
         <v>13</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C14" s="9"/>
-      <c r="D14" s="9" t="s">
-        <v>217</v>
-      </c>
+      <c r="D14" s="9"/>
       <c r="E14" s="9" t="s">
         <v>218</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>95</v>
+        <v>219</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>219</v>
+        <v>96</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>220</v>
@@ -3837,14 +3888,17 @@
       <c r="L14" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="M14" s="11">
+      <c r="M14" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="N14" s="11">
         <v>0.72</v>
       </c>
-      <c r="N14" s="9" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="409.6">
+      <c r="O14" s="9" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="409.6">
       <c r="A15" s="9">
         <v>14</v>
       </c>
@@ -3852,17 +3906,15 @@
         <v>60</v>
       </c>
       <c r="C15" s="9"/>
-      <c r="D15" s="9" t="s">
-        <v>226</v>
-      </c>
+      <c r="D15" s="9"/>
       <c r="E15" s="9" t="s">
         <v>227</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>95</v>
+        <v>228</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>228</v>
+        <v>96</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>229</v>
@@ -3879,32 +3931,33 @@
       <c r="L15" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="M15" s="11">
+      <c r="M15" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="N15" s="11">
         <v>0.9</v>
       </c>
-      <c r="N15" s="9" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="396.75">
+      <c r="O15" s="9" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="396.75">
       <c r="A16" s="9">
         <v>15</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C16" s="9"/>
-      <c r="D16" s="9" t="s">
-        <v>186</v>
-      </c>
+      <c r="D16" s="9"/>
       <c r="E16" s="9" t="s">
-        <v>236</v>
+        <v>187</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>187</v>
+        <v>237</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>237</v>
+        <v>188</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>238</v>
@@ -3921,34 +3974,35 @@
       <c r="L16" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="M16" s="11">
+      <c r="M16" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="N16" s="11">
         <v>0.93</v>
       </c>
-      <c r="N16" s="9" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="321">
+      <c r="O16" s="9" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="321">
       <c r="A17" s="9">
         <v>16</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="D17" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="E17" s="9">
+      <c r="D17" s="9"/>
+      <c r="E17" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="F17" s="9">
         <v>1962</v>
       </c>
-      <c r="F17" s="9" t="s">
-        <v>187</v>
-      </c>
       <c r="G17" s="9" t="s">
-        <v>247</v>
+        <v>188</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>248</v>
@@ -3965,14 +4019,17 @@
       <c r="L17" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="M17" s="11">
+      <c r="M17" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="N17" s="11">
         <v>0.9</v>
       </c>
-      <c r="N17" s="9" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="381.75">
+      <c r="O17" s="9" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="381.75">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -3980,19 +4037,17 @@
         <v>67</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="D18" s="9" t="s">
         <v>255</v>
       </c>
+      <c r="D18" s="9"/>
       <c r="E18" s="9" t="s">
         <v>256</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>187</v>
+        <v>257</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>257</v>
+        <v>188</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>258</v>
@@ -4009,32 +4064,32 @@
       <c r="L18" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="M18" s="11">
+      <c r="M18" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="N18" s="11">
         <v>0.91</v>
       </c>
-      <c r="N18" s="9" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="409.6">
+      <c r="O18" s="9" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="409.6">
       <c r="A19" s="9">
         <v>18</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C19" t="s">
-        <v>265</v>
-      </c>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9" t="s">
         <v>266</v>
       </c>
+      <c r="E19" s="9"/>
       <c r="F19" s="9" t="s">
-        <v>95</v>
+        <v>267</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>267</v>
+        <v>96</v>
       </c>
       <c r="H19" s="9" t="s">
         <v>268</v>
@@ -4051,32 +4106,33 @@
       <c r="L19" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="M19" s="11">
+      <c r="M19" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="N19" s="11">
         <v>0.95</v>
       </c>
-      <c r="N19" s="9" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="396.75">
+      <c r="O19" s="9" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="396.75">
       <c r="A20" s="9">
         <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D20" s="9"/>
-      <c r="E20" s="9" t="s">
-        <v>218</v>
-      </c>
+      <c r="E20" s="9"/>
       <c r="F20" s="9" t="s">
-        <v>95</v>
+        <v>219</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>276</v>
+        <v>96</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>277</v>
@@ -4093,32 +4149,33 @@
       <c r="L20" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="M20" s="11">
+      <c r="M20" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="N20" s="11">
         <v>0.95</v>
       </c>
-      <c r="N20" s="9" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="366">
+      <c r="O20" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="366">
       <c r="A21" s="9">
         <v>20</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
-      <c r="E21" s="9" t="s">
-        <v>284</v>
-      </c>
+      <c r="E21" s="9"/>
       <c r="F21" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="G21" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="G21" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="H21" s="1" t="s">
         <v>286</v>
       </c>
       <c r="I21" s="9" t="s">
@@ -4133,11 +4190,14 @@
       <c r="L21" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="M21" s="11">
+      <c r="M21" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="N21" s="11">
         <v>0.86</v>
       </c>
-      <c r="N21" s="9" t="s">
-        <v>291</v>
+      <c r="O21" s="9" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -4162,23 +4222,23 @@
         <v>78</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="381.75">
       <c r="A2" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="381.75">
       <c r="A3" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="366">
@@ -4186,15 +4246,15 @@
         <v>26</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="91.5">
       <c r="A5" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="381.75">
@@ -4202,71 +4262,71 @@
         <v>38</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="91.5">
       <c r="A7" s="9" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="106.5">
       <c r="A8" s="9" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="76.5">
       <c r="A9" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="152.25">
       <c r="A10" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="183">
       <c r="A11" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="91.5">
       <c r="A12" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="91.5">
       <c r="A13" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="76.5">
       <c r="A14" s="9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="91.5">
@@ -4274,23 +4334,23 @@
         <v>60</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="91.5">
       <c r="A16" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="76.5">
       <c r="A17" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="91.5">
@@ -4298,31 +4358,31 @@
         <v>67</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="91.5">
       <c r="A19" s="9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="91.5">
       <c r="A20" s="9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="76.5">
       <c r="A21" s="9" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: improve vision prompt and search pipeline
- redesign Vision prompt to reduce feature inference
- add structured visual features (frame geometry, armrests, supports)
- migrate search to English search_features
- improve SQLite import with reference_id support
- update reference images for core furniture models
- improve search scoring and verification pipeline
- add debug logging for Vision, Search and Verification
</commit_message>
<xml_diff>
--- a/data/furniture.xlsx
+++ b/data/furniture.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B691E158-FE89-466B-8953-B0ED820191F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{21A469CB-CEF7-437C-AD60-690DE7A566ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="298">
   <si>
     <t>Prompt 1</t>
   </si>
@@ -353,6 +353,681 @@
   </si>
   <si>
     <t>opracowania dotyczące Józefa Chierowskiego; dokumentacja 366 Concept; zbiory Muzeum Narodowego w Warszawie; Polski New Look Ewa Solarz i Agnieszka Sural; publikacje o polskim wzornictwie powojennym</t>
+  </si>
+  <si>
+    <t>armchair;
+wooden frame;
+open frame;
+a-frame side construction;
+triangular side frame;
+angled front support;
+flat plank armrests;
+rounded wooden armrests;
+wide wooden armrests;
+visible screw joints;
+tapered wooden legs;
+splayed legs;
+floating seat;
+rounded box seat cushion;
+rounded rectangular backrest;
+slightly reclined backrest;
+button tufting;
+integrated seat and backrest;
+open space under seat;
+exposed wooden structure;
+organic armrest shape;</t>
+  </si>
+  <si>
+    <t>Fotel typ 300-190</t>
+  </si>
+  <si>
+    <t>Lisek</t>
+  </si>
+  <si>
+    <t>Henryk Lis</t>
+  </si>
+  <si>
+    <t>Dolnośląska Fabryka Mebli w Świebodzicach; Bystrzyckie Fabryki Mebli; Zakład Mebli Giętych FAMEG Radomsko; Świdnicki Ośrodek Przemysłu Meblarskiego</t>
+  </si>
+  <si>
+    <t>Fotel posiada lekką, smukłą konstrukcję opartą na odsłoniętej drewnianej ramie. Tapicerowane siedzisko i oparcie osadzone są pomiędzy drewnianymi boczkami zakończonymi płaskimi podłokietnikami. Konstrukcja wsparta jest na czterech toczonych, lekko zwężających się nogach. W połowie wysokości nóg widoczne są poprzeczne belki tworzące charakterystyczną ramę usztywniającą. Drewniane elementy wykończone były lakierem o wykończeniu matowym, półmatowym lub z połyskiem.</t>
+  </si>
+  <si>
+    <t>Konstrukcję nośną tworzą drewniane boczki połączone poprzecznymi belkami oraz stelażem. Nogi są mocowane do płaskich podłokietników. Do wykonania stolarki zastosowano drewno bukowe. Siedzisko wykorzystuje formatki gumowe osadzone na elastycznych pasach zamiast sprężyn i tradycyjnych wypełnień.</t>
+  </si>
+  <si>
+    <t>typ 366; GFM-64; fotele klubowe PRL z lat 60.</t>
+  </si>
+  <si>
+    <t>zestaw Odra; zestaw Syrena; warianty produkcyjne różnych fabryk (Do weryfikacji)</t>
+  </si>
+  <si>
+    <t>Nowohuckie Renowacje – Fotel Lisek typ 300-190; Conchita Home – 4 fotele z PRL które musisz znać; dokumentacja i opisy egzemplarzy Typ 300-190; archiwalne materiały producentów cytowane w opracowaniach specjalistycznych</t>
+  </si>
+  <si>
+    <t>armchair;
+wooden frame;
+open frame;
+rectangular side frame;
+horizontal lower stretcher;
+flat plank armrests;
+long narrow armrests;
+rounded armrest ends;
+vertical front support;
+angled rear support;
+tapered wooden legs;
+slightly splayed legs;
+floating upholstered seat;
+box seat cushion;
+tall rectangular backrest;
+slightly reclined backrest;
+thin side profile;
+lightweight construction;
+visible wooden frame;
+open space under seat;
+straight geometric lines;
+minimalist frame;
+visible side rails;
+parallel armrests;
+rectangular geometry;
+exposed wooden structure;</t>
+  </si>
+  <si>
+    <t>Do weryfikacji; często błędnie określany jako „Lisek”</t>
+  </si>
+  <si>
+    <t>Henryk Lis (do potwierdzenia)</t>
+  </si>
+  <si>
+    <t>1969–1970</t>
+  </si>
+  <si>
+    <t>Zakłady Przemysłu Meblarskiego im. Gwardii Ludowej w Radomsku; Fabryki Mebli Radomsko</t>
+  </si>
+  <si>
+    <t>Fotel posiada otwartą drewnianą konstrukcję zewnętrzną wykonaną z litego drewna. Tapicerowane siedzisko i oparcie zamocowane są wewnątrz drewnianej ramy za pomocą wkrętów lub śrub. Konstrukcja opiera się na czterech toczonych nogach połączonych belkami podtrzymującymi siedzisko. Charakterystycznym elementem są zaokrąglone drewniane podłokietniki stanowiące integralną część bocznej ramy.</t>
+  </si>
+  <si>
+    <t>Konstrukcja wykonana jest z litej tarcicy bukowej. Szkielet ukryty pod tapicerką wykonano z tarcicy iglastej. Siedzisko i oparcie mocowane są do ramy za pomocą wkrętów lub śrub. Połączenia konstrukcyjne obejmują połączenia czopowe oraz połączenia na wkręty. W siedzisku zastosowano pasy tapicerskie i tworzywo piankowe.</t>
+  </si>
+  <si>
+    <t>typ 300-190 Lisek; BW-14; typ 366</t>
+  </si>
+  <si>
+    <t>rodzina foteli Radomsko o otwartej konstrukcji ramowej; BW-14; typ 300-190 Lisek (wizualnie pokrewny)</t>
+  </si>
+  <si>
+    <t>Patyna.pl – fotel B-7727 Radomsko PRL; Meblostan – fotel B-7727; Nowohuckie Renowacje – fotel B-7727; Vilandy – fotel Lis typ B-7727; Allegro – fotel PRL model B-7727 Radomsko lata 70; Reko-Czyny – identyfikacja fotela B-7727</t>
+  </si>
+  <si>
+    <t>wooden frame;
+open frame;
+rectangular side frame;
+floating seat;
+floating backrest;
+separate seat cushion;
+separate backrest;
+box seat cushion;
+tall rectangular backrest;
+slightly reclined backrest;
+rounded plank armrests;
+wide rounded armrests;
+thick armrests;
+rounded armrest ends;
+curved armrest profile;
+vertical front support;
+angled rear support;
+horizontal lower stretcher;
+tapered wooden legs;
+slightly splayed legs;
+rounded wooden posts;
+visible screw joints;
+visible frame connections;
+solid wooden frame;
+heavier frame;
+robust construction;
+visible wooden side rails;
+open space under seat;</t>
+  </si>
+  <si>
+    <t>Typ 300-177</t>
+  </si>
+  <si>
+    <t>Bunny; Zajączek</t>
+  </si>
+  <si>
+    <t>Józef Chierowski (Do weryfikacji – atrybucja często powtarzana w źródłach kolekcjonerskich, słabo potwierdzona w publikacjach naukowych)</t>
+  </si>
+  <si>
+    <t>początek lat 60. XX w.</t>
+  </si>
+  <si>
+    <t>Świebodzińskie Fabryki Mebli; Gościcińskie Fabryki Mebli</t>
+  </si>
+  <si>
+    <t>trójkątne podłokietniki; lekka drewniana konstrukcja; kompaktowe wymiary; szeroko rozstawione nogi; tapicerowane siedzisko i oparcie; forma nawiązująca do modelu 366</t>
+  </si>
+  <si>
+    <t>bukowy stelaż; otwarta konstrukcja boczna; tapicerowane moduły siedziska i oparcia; drewniane podłokietniki zintegrowane z ramą; konstrukcja szkieletowa</t>
+  </si>
+  <si>
+    <t>typ 366; typ 300-190 Lisek; BW-14</t>
+  </si>
+  <si>
+    <t>typ 366; grupa lekkich foteli drewnianych PRL z lat 60.; modele produkowane przez Świebodzińskie i Gościcińskie Fabryki Mebli (Do weryfikacji)</t>
+  </si>
+  <si>
+    <t>Meblostan – Fotel Bunny typ 300-177; Nowohuckie Renowacje – Fotel typ 300-177 Zajączek; Patyna.pl – Fotel Bunny typ 300-177; Tkaniny-Meblowe.pl – Fotele z PRL-u; materiały kolekcjonerskie rynku vintage</t>
+  </si>
+  <si>
+    <t>trójkątne podłokietniki przypominające uszy zająca; otwarta drewniana rama boczna; szeroko rozstawione nogi; podłokietniki połączone z przednimi nogami; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; smukła lekka bryła; odsłonięty drewniany stelaż; skośne tylne nogi; geometryczny profil boczny; kompaktowe proporcje</t>
+  </si>
+  <si>
+    <t>Fotel Ewa; Muszelka Ewa</t>
+  </si>
+  <si>
+    <t>Do weryfikacji</t>
+  </si>
+  <si>
+    <t>Strzeleckie Zakłady Przemysłu Terenowego w Strzelcach Opolskich</t>
+  </si>
+  <si>
+    <t>Fotel posiada muszelkowy, kubełkowy korpus tworzący jednolitą tapicerowaną bryłę. Szerokie, półkoliste oparcie płynnie przechodzi w siedzisko, nadając bryle profil przypominający muszlę. Korpus osadzony jest na odsłoniętym stalowym stelażu wspartym na czterech smukłych metalowych nogach. Fotel nie posiada drewnianych podłokietników, a wysoka podstawa nadaje konstrukcji lekką formę.</t>
+  </si>
+  <si>
+    <t>Konstrukcję nośną stanowi rama wykonana ze spawanych prętów stalowych. Rama wsparta jest na czterech stalowych, wykręcanych nogach zakończonych ruchomymi stopkami. W modelu Koeln 1 zastosowano pojedynczą stalową nogę obrotową.</t>
+  </si>
+  <si>
+    <t>fotel Köln 1; fotel Muszelka; fotele klubowe na stelażu stalowym z lat 60.</t>
+  </si>
+  <si>
+    <t>Köln 1 (NRD); fotele muszelkowe PRL; metalowe fotele klubowe lat 60.</t>
+  </si>
+  <si>
+    <t>Meblostan – Para foteli tapicerowanych EWA; Odnowa Mebli – Fotel Ewa; Patyna.pl – Komplet foteli typ Ewa; materiały kolekcjonerskie rynku vintage</t>
+  </si>
+  <si>
+    <t>rounded_shell;
+bucket_seat;
+integrated_shell;
+one_piece_body;
+continuous_backrest;
+continuous_armrests;
+curved_side_profile;
+organic_shape;
+wide_rounded_backrest;
+rounded_top_backrest;
+high_backrest;
+integrated_armrests;
+wrapped_armrests;
+upholstered_shell;
+soft_shell;
+floating_shell;
+metal_frame;
+steel_frame;
+four_metal_legs;
+slender_metal_legs;
+slightly_splayed_legs;
+black_metal_legs;
+metal_feet;
+round_feet_caps;
+open_space_under_shell;
+no_wooden_frame;
+no_wooden_armrests;
+lightweight_construction;
+minimalist_design;</t>
+  </si>
+  <si>
+    <t>Typ 300-123</t>
+  </si>
+  <si>
+    <t>Puchała; wersja damska (Do weryfikacji)</t>
+  </si>
+  <si>
+    <t>Mieczysław Puchała</t>
+  </si>
+  <si>
+    <t>1956 (według części źródeł); początek lat 60. XX w.</t>
+  </si>
+  <si>
+    <t>lekka smukła sylwetka; gięte drewniane podłokietniki; wysokie oparcie; wąskie proporcje; odsłonięta drewniana konstrukcja; toczone nogi; modernistyczna forma inspirowana wzornictwem skandynawskim</t>
+  </si>
+  <si>
+    <t>drewniany stelaż bukowy; otwarta konstrukcja boczna; tapicerowane siedzisko; tapicerowane oparcie; pasy tapicerskie; konstrukcja szkieletowa</t>
+  </si>
+  <si>
+    <t>typ 300-137; typ 300-190 Lisek; typ 366</t>
+  </si>
+  <si>
+    <t>typ 300-137 wersja męska; rodzina foteli projektu Mieczysława Puchały; lekkie fotele drewniane PRL lat 50. i 60</t>
+  </si>
+  <si>
+    <t>Nowohuckie Renowacje – Fotel typ 300-123 Puchała; Szajba Sklep – Fotel klubowy typ 300-123 proj. M. Puchała; LookInside – Fotel typ 300-123 Puchała; Pakamera – Fotel typ 300-123 M. Puchała; Meblostan – Fotel Puchały typ 300-123</t>
+  </si>
+  <si>
+    <t>gięte drewniane podłokietniki; smukłe wysokie oparcie; wąskie proporcje korpusu; otwarta drewniana rama boczna; toczone nogi zwężające się ku dołowi; widoczny prześwit pod siedziskiem; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; lekka dynamiczna bryła; cienkie elementy konstrukcyjne; profil boczny z łukowato wygiętym podłokietnikiem; minimalistyczna forma lat 50./60.</t>
+  </si>
+  <si>
+    <t>RM58</t>
+  </si>
+  <si>
+    <t>Muszelka; RM58</t>
+  </si>
+  <si>
+    <t>Roman Modzelewski</t>
+  </si>
+  <si>
+    <t>Zakłady Mebli Artystycznych w Łodzi (prototyp); Vzór Sp. z o.o. (reedycja od 2012 r.)</t>
+  </si>
+  <si>
+    <t>organiczna muszelkowa forma; jednolita zamknięta bryła; głębokie kubełkowe siedzisko; szerokie wywinięte boki; opływowy futurystyczny kształt; brak klasycznych podłokietników; rzeźbiarska sylwetka</t>
+  </si>
+  <si>
+    <t>jednoczęściowy korpus z laminatu poliestrowo-szklanego; tapicerowana wkładka siedziska; cztery smukłe nogi; technologia laminatu wyprzedzająca epokę w Polsce; konstrukcja skorupowa</t>
+  </si>
+  <si>
+    <t>fotel Ewa; fotele muszelkowe produkcji NRD; zachodnie fotele fiberglass lat 50.; projekty Eero Saarinena</t>
+  </si>
+  <si>
+    <t>prototypowe meble z laminatu Romana Modzelewskiego; współczesne reedycje RM58; warianty kolorystyczne RM58 Classic</t>
+  </si>
+  <si>
+    <t>Muzeum Narodowe we Wrocławiu; Vzór – dokumentacja reedycji RM58; Instytut Wzornictwa Przemysłowego; publikacje o twórczości Romana Modzelewskiego; Culture.pl</t>
+  </si>
+  <si>
+    <t>jednoczęściowa muszelkowa skorupa; organiczna opływowa bryła; głębokie kubełkowe siedzisko; szerokie wywinięte boki; zaokrąglone wysokie oparcie; brak oddzielnych podłokietników; korpus przypominający muszlę; zamknięta forma boczna; cztery cienkie nogi; futurystyczna sylwetka lat 50.; brak widocznej drewnianej konstrukcji; płynne przejścia między siedziskiem i oparciem; asymetrycznie zaokrąglone krawędzie; korpus wykonany jako pojedyncza skorupa</t>
+  </si>
+  <si>
+    <t>B-2020</t>
+  </si>
+  <si>
+    <t>Tulipan</t>
+  </si>
+  <si>
+    <t>Teresa Kruszewska</t>
+  </si>
+  <si>
+    <t>1973 (prototyp)</t>
+  </si>
+  <si>
+    <t>FAMEG Radomsko (reedycja współczesna)</t>
+  </si>
+  <si>
+    <t>organiczna forma inspirowana kielichem kwiatu; szerokie kubełkowe siedzisko; płynne przejście między siedziskiem i oparciem; miękkie zaokrąglone linie; wyraźnie rozchylone boki; rzeźbiarska bryła</t>
+  </si>
+  <si>
+    <t>korpus ze sklejki formowanej; tapicerowana skorupa; drewniana podstawa; konstrukcja monolityczna; technologia giętej sklejki</t>
+  </si>
+  <si>
+    <t>RM58; fotele muszelkowe PRL; fotele skandynawskie o organicznej formie</t>
+  </si>
+  <si>
+    <t>projekty Teresy Kruszewskiej; meble ze sklejki formowanej; współczesna kolekcja Tulipan FAMEG</t>
+  </si>
+  <si>
+    <t>FAMEG – Fotel Tulipan B-2020; dokumentacja reedycji FAMEG; opracowania dotyczące twórczości Teresy Kruszewskiej</t>
+  </si>
+  <si>
+    <t>kubełkowe siedzisko; forma przypominająca kielich tulipana; szeroko rozchylone boki; jednolita tapicerowana skorupa; zaokrąglone wysokie oparcie; płynne przejście między siedziskiem i oparciem; organiczna bryła; brak widocznej drewnianej ramy bocznej; miękkie obłe krawędzie; rzeźbiarska forma; kompaktowa podstawa; sylwetka kwiatu tulipana</t>
+  </si>
+  <si>
+    <t>Typ 300-201</t>
+  </si>
+  <si>
+    <t>Śnieżnik; Śnieżka (Do weryfikacji – obie nazwy występują w obiegu kolekcjonerskim, częściej spotykana jest nazwa Śnieżnik)</t>
+  </si>
+  <si>
+    <t>1973 (najwcześniejsza potwierdzona wzmianka źródłowa)</t>
+  </si>
+  <si>
+    <t>Bystrzycka Fabryka Mebli w Bystrzycy Kłodzkiej</t>
+  </si>
+  <si>
+    <t>lekka konstrukcja drewniana; forma inspirowana modelem Lisek 300-190; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; otwarta rama boczna; charakterystyczne nogi częściowo graniaste i częściowo zaokrąglone; smukłe proporcje</t>
+  </si>
+  <si>
+    <t>drewniany stelaż brzozowy lub bukowy; otwarta konstrukcja boczna; tapicerowane siedzisko; tapicerowane oparcie; pasy tapicerskie; konstrukcja szkieletowa</t>
+  </si>
+  <si>
+    <t>typ 300-190 Lisek; Śnieżka; BW-14 typ 300-199; B-7727</t>
+  </si>
+  <si>
+    <t>typ 300-190 Lisek; Śnieżka; BW-14 typ 300-199; BW-20 typ 300-193; B-7727</t>
+  </si>
+  <si>
+    <t>Meblostan – Fotel Śnieżnik typ 300-201; Nowohuckie Renowacje – Fotele PRL; Pakamera – Fotel Śnieżnik typ 300-201; Audiovintage Store – Fotel klubowy Śnieżnik 300-201</t>
+  </si>
+  <si>
+    <t>otwarta drewniana rama boczna; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; smukła lekka bryła; duży prześwit pod siedziskiem; drewniane podłokietniki zintegrowane z ramą; nogi graniaste od góry; nogi zaokrąglone w dolnej części; skośne tylne nogi; widoczne drewniane elementy konstrukcyjne; forma zbliżona do modelu Lisek; geometryczny profil boczny
+Źródła potwierdzają produkcję w Bystrzyckiej Fabryce Mebli oraz silne pokrewieństwo konstrukcyjne z modelem 300-190 „Lisek”, natomiast projektant pozostaje niepotwierdzony.</t>
+  </si>
+  <si>
+    <t>GFM-57</t>
+  </si>
+  <si>
+    <t>Skoczek</t>
+  </si>
+  <si>
+    <t>Juliusz Kędziorek</t>
+  </si>
+  <si>
+    <t>Krzesło</t>
+  </si>
+  <si>
+    <t>Gościcińska Fabryka Mebli; Zamojskie Fabryki Mebli (produkcja seryjna jako typ 200-203)</t>
+  </si>
+  <si>
+    <t>łukowate podłokietniki przypominające profil skoczni narciarskiej; elipsoidalne oparcie; lekka ażurowa konstrukcja; zwężające się ku dołowi nogi; tapicerowane siedzisko; smukła sylwetka; organiczna linia boczna</t>
+  </si>
+  <si>
+    <t>drewniany stelaż; otwarta konstrukcja boczna; tapicerowane siedzisko; gięte elementy drewniane; konstrukcja przeznaczona do produkcji seryjnej</t>
+  </si>
+  <si>
+    <t>typ 200-190 Rajmunda Hałasa; krzesła Aga; krzesła patyczaki lat 60.; lekkie krzesła tapicerowane PRL</t>
+  </si>
+  <si>
+    <t>typ 200-203; GFM-107; projekty Juliusza Kędziorka dla Gościcińskiej Fabryki Mebli</t>
+  </si>
+  <si>
+    <t>Magazif – Krzesło Skoczek; Ikony Designu PL – Krzesło GFM-57 Skoczek; Meblostan – Krzesło Skoczek; Sosenko Home Decor – Krzesło Skoczek; Allegro Artykuł – Krzesło kilka słów o najtrudniejszym meblu</t>
+  </si>
+  <si>
+    <t>łukowate podłokietniki przypominające skocznię narciarską; elipsoidalne oparcie; otwarta drewniana rama boczna; smukłe zwężające się nogi; tapicerowane siedzisko; duży prześwit pod siedziskiem; płynna linia podłokietnika przechodząca w nogę; lekka ażurowa konstrukcja; organiczny profil boczny; oparcie w kształcie pionowej elipsy; cienkie elementy drewniane; dynamiczna sylwetka inspirowana skokami narciarskimi
+Źródła potwierdzają, że model został zaprojektowany przez Juliusza Kędziorka w Gościcińskiej Fabryce Mebli w 1965 r., otrzymał nagrodę „Dobre–Ładne–Poszukiwane” i został skierowany do produkcji seryjnej jako typ 200-203</t>
+  </si>
+  <si>
+    <t>Typ 200-125 VAR</t>
+  </si>
+  <si>
+    <t>Aga</t>
+  </si>
+  <si>
+    <t>ok. 1972–1975 (w źródłach występują rozbieżności dotyczące dokładnego roku projektu)</t>
+  </si>
+  <si>
+    <t>Wielkopolskie Fabryki Mebli; produkcja seryjna PRL (pozostali producenci wymagają weryfikacji)</t>
+  </si>
+  <si>
+    <t>wysokie tapicerowane oparcie; trapezowy układ nóg; miękkie tapicerowane siedzisko; smukła skandynawska forma; zwężająca się ku górze bryła; lekkie proporcje; drewniana konstrukcja eksponowana po bokach</t>
+  </si>
+  <si>
+    <t>drewniany stelaż bukowy; tapicerowane siedzisko; tapicerowane oparcie; sprężyny siedziska; cztery drewniane nogi; konstrukcja przeznaczona do intensywnego użytkowania klubowego</t>
+  </si>
+  <si>
+    <t>typ 200-190 Rajmunda Hałasa; GFM-57 Skoczek; lekkie krzesła klubowe PRL lat 70.</t>
+  </si>
+  <si>
+    <t>fotel 366; meble klubowe Józefa Chierowskiego; reedycja 200-125 VAR realizowana przez 366 Concept</t>
+  </si>
+  <si>
+    <t>Elle Decoration Polska – Krzesło VAR AGA projektu Józefa Chierowskiego; Nowohuckie Renowacje – Krzesło Aga typ 200-125; Patyna.pl – Krzesła AGA typu 200-125 VAR; Linie Studio – 200-125 VAR; Meblościanka – 200-125 VAR</t>
+  </si>
+  <si>
+    <t>wysokie tapicerowane oparcie; trapezowy układ nóg; szerokie miękkie siedzisko; brak podłokietników; drewniane nogi rozszerzające się ku dołowi; zwężająca się ku górze sylwetka; lekka skandynawska forma; prostokątne oparcie z zaokrąglonymi krawędziami; widoczne drewniane elementy boczne; smukłe proporcje; geometryczna bryła; profil boczny z pochylonym oparciem</t>
+  </si>
+  <si>
+    <t>Typ 200-190</t>
+  </si>
+  <si>
+    <t>Hałas; Grzybek</t>
+  </si>
+  <si>
+    <t>Rajmund Teofil Hałas</t>
+  </si>
+  <si>
+    <t>lata 60. XX w.; dokładny rok projektu – Do weryfikacji</t>
+  </si>
+  <si>
+    <t>Zakłady Mebli w Gostyniu (Do weryfikacji); produkcja seryjna w kilku zakładach meblarskich PRL – Do weryfikacji</t>
+  </si>
+  <si>
+    <t>okrągła forma oparcia przypominająca kapelusz grzyba; tapicerowane oparcie i siedzisko; smukłe zwężające się nogi; lekka konstrukcja; wyraźnie wyodrębnione oparcie nad siedziskiem; proporcje inspirowane wzornictwem skandynawskim; minimalistyczna sylwetka</t>
+  </si>
+  <si>
+    <t>drewniany stelaż; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; mocowane oddzielnie siedzisko i oparcie; nogi zwężające się ku dołowi</t>
+  </si>
+  <si>
+    <t>Aga 200-125; Skoczek GFM-57; krzesła skandynawskie lat 60.; lekkie krzesła tapicerowane PRL</t>
+  </si>
+  <si>
+    <t>projekty Rajmunda Teofila Hałasa; krzesła tapicerowane PRL lat 60.; warianty produkcyjne typu 200-190</t>
+  </si>
+  <si>
+    <t>Odnawialnia – Wiem co odnawiam | krzesło Hałasa typ 200-190; Patyna.pl – Krzesła typ 200-190 Rajmund Teofil Hałas; Meblostan – Komplet krzeseł typ 200-190; Daniel Stoiński Redesign – Przewodnik po renowacji krzesła 200-190; Homebook – Krzesło Hałasa typ 200-190</t>
+  </si>
+  <si>
+    <t>okrągłe oparcie przypominające grzybek; oparcie szersze od wspornika; tapicerowane okrągłe oparcie; tapicerowane siedzisko; smukłe nogi zwężające się ku dołowi; brak podłokietników; lekka skandynawska forma; duży prześwit pod siedziskiem; cienki drewniany stelaż; wyraźne oddzielenie oparcia od siedziska; geometryczna bryła; profil boczny z lekko odchylonym oparciem</t>
+  </si>
+  <si>
+    <t>B-6028</t>
+  </si>
+  <si>
+    <t>Barbara Fenrych-Węcławska (Do weryfikacji); Józef Chierowski (Do weryfikacji – atrybucja pojawiająca się wyłącznie w źródłach kolekcjonerskich)</t>
+  </si>
+  <si>
+    <t>lata 60. XX w.</t>
+  </si>
+  <si>
+    <t>Fabryka Mebli Giętych w Radomsku; FAMEG Radomsko; Radomszczańska Fabryka Mebli Giętych</t>
+  </si>
+  <si>
+    <t>wysokie profilowane oparcie; szerokie drewniane podłokietniki; gięte elementy bukowe; głębokie siedzisko; lekka otwarta konstrukcja boczna; elegancka smukła sylwetka; forma łącząca cechy fotela klubowego i wypoczynkowego</t>
+  </si>
+  <si>
+    <t>stelaż z giętego drewna bukowego; otwarta konstrukcja ramowa; tapicerowane siedzisko; tapicerowane oparcie; drewniane podłokietniki zintegrowane z ramą; konstrukcja szkieletowa</t>
+  </si>
+  <si>
+    <t>typ 300-123 Puchała; typ 300-177 Zajączek; B-7727; typ 366</t>
+  </si>
+  <si>
+    <t>fotele Radomsko z giętego drewna; projekty Barbary Fenrych-Węcławskiej (Do weryfikacji); lekkie fotele klubowe PRL lat 60.</t>
+  </si>
+  <si>
+    <t>MidMod – Fotel B6028 FAMEG Radomsko Polska lata 60; Oldsen Design – Fotel B6028 prod. FAMEG Radomsko; Nowohuckie Renowacje – Fotel PRL B-6028 z lat 60-tych; Fotelowo Facebook – fotel projektu Barbary Fenrych-Węcławskiej; Instagram Renowacja Mebli PRL – B6028 lata produkcji 1960</t>
+  </si>
+  <si>
+    <t>wysokie prostokątne oparcie; szerokie drewniane podłokietniki; gięte boczne elementy z drewna; otwarta rama boczna; głębokie siedzisko; masywniejsza bryła niż typ 366; bukowy stelaż; duży prześwit pod siedziskiem; profilowane podłokietniki; smukłe nogi zintegrowane z ramą; tapicerowane oparcie i siedzisko; geometryczny profil boczny</t>
+  </si>
+  <si>
+    <t>A. Dutka</t>
+  </si>
+  <si>
+    <t>1966–1968</t>
+  </si>
+  <si>
+    <t>Zakłady Mebli Giętych w Radomsku; Gołuchowskie Fabryki Mebli</t>
+  </si>
+  <si>
+    <t>duże gabaryty; szerokie głębokie siedzisko; masywne drewniane podłokietniki; geometryczna forma boczna; lekko pochylone oparcie; otwarta konstrukcja ramowa; modernistyczna sylwetka eksportowa</t>
+  </si>
+  <si>
+    <t>stelaż z drewna bukowego; sprężyny lejowe w siedzisku; tapicerowane siedzisko i oparcie; otwarta konstrukcja boczna; drewniane podłokietniki zintegrowane z ramą; konstrukcja rozbieralna skręcana śrubami</t>
+  </si>
+  <si>
+    <t>B-6028; GFM-64; typ 300-190 Lisek; B-7727</t>
+  </si>
+  <si>
+    <t>fotele eksportowe Radomsko lat 60.; modele Zakładów Mebli Giętych w Radomsku; konstrukcje projektowane przez A. Dutkę (Do weryfikacji)</t>
+  </si>
+  <si>
+    <t>Meblostan – Para foteli B-310 VAR; Pufa Design – Oryginalny fotel B-310 VAR; Yestersen – Fotel B-310 VAR Polska lata 70.; Reko-Czyny – Fotel B-310 VAR metamorfoza; archiwalne ogłoszenia kolekcjonerskie B-310 VAR</t>
+  </si>
+  <si>
+    <t>masywne drewniane podłokietniki; szerokie głębokie siedzisko; wysunięte przednie podłokietniki; otwarta drewniana rama boczna; prostokątne tapicerowane oparcie; grube proporcje siedziska; lekko pochylone oparcie; duży prześwit pod siedziskiem; widoczne śruby montażowe w ramie; geometryczny profil boczny; szeroki rozstaw nóg; cięższa bryła niż typ 366; bukowy stelaż; modernistyczna forma eksportowa</t>
+  </si>
+  <si>
+    <t>GFM-22 (typ 200/128)</t>
+  </si>
+  <si>
+    <t>ok. 1960</t>
+  </si>
+  <si>
+    <t>Gościcińska Fabryka Mebli (GFM)</t>
+  </si>
+  <si>
+    <t>nerkowate oparcie; lekka ażurowa konstrukcja; smukłe zwężające się nogi; gięta drewniana rama; tapicerowane siedzisko; tapicerowane oparcie; wyraźnie rozstawione tylne nogi</t>
+  </si>
+  <si>
+    <t>drewniany stelaż; gięte elementy z litego drewna; tapicerowane siedzisko; tapicerowane oparcie ze sklejki giętej; konstrukcja szkieletowa przeznaczona do produkcji seryjnej</t>
+  </si>
+  <si>
+    <t>GFM-57 Skoczek; typ 200-190 Rajmunda Hałasa; Aga 200-125; krzesła skandynawskie z lat 60.</t>
+  </si>
+  <si>
+    <t>typ 200/128; projekty Juliusza Kędziorka dla Gościcińskiej Fabryki Mebli; GFM-57; GFM-87</t>
+  </si>
+  <si>
+    <t>Pamono – Mid-Century GFM-22 Chairs by Juliusz Kędziorek; Vinterior – GFM-22 model 200/128; Selency – Iconic GFM-22 Chair by Juliusz Kędziorek; Instagram Zostań z Vintage – Krzesło GFM-22 typ 200/128</t>
+  </si>
+  <si>
+    <t>nerkowate tapicerowane oparcie; oparcie szersze od wspornika; smukłe zwężające się nogi; lekka ażurowa konstrukcja; gięta drewniana rama; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; cienkie elementy konstrukcyjne; szeroko rozstawione tylne nogi; profil boczny z delikatnie pochylonym oparciem; organiczny kształt oparcia; minimalistyczna sylwetka lat 60.</t>
+  </si>
+  <si>
+    <t>Typ 1020</t>
+  </si>
+  <si>
+    <t>Muszelka</t>
+  </si>
+  <si>
+    <t>Wiesław Leśniewski; Stanisław Lejkowski</t>
+  </si>
+  <si>
+    <t>Słupskie Fabryki Mebli</t>
+  </si>
+  <si>
+    <t>muszelkowe profilowane oparcie; jednolita tapicerowana skorupa; zaokrąglona górna krawędź oparcia; smukłe stożkowe nogi; lekka modernistyczna forma; brak podłokietników; organiczna sylwetka</t>
+  </si>
+  <si>
+    <t>profilowana skorupa ze sklejki; tapicerowana skorupa; drewniany stelaż; cztery drewniane nogi; konstrukcja szkieletowa; połączenie sklejki i drewna litego</t>
+  </si>
+  <si>
+    <t>RM58; krzesła muszelkowe produkcji NRD; krzesła skandynawskie lat 60.; fotel Ewa</t>
+  </si>
+  <si>
+    <t>krzesła muszelkowe Słupskich Fabryk Mebli; projekty Wiesława Leśniewskiego i Stanisława Lejkowskiego; meble ze sklejki profilowanej produkowane przez SFM</t>
+  </si>
+  <si>
+    <t>Archiwalne katalogi Słupskich Fabryk Mebli; opracowania kolekcjonerskie dotyczące wzornictwa SFM; materiały renowatorów specjalizujących się w meblach PRL; publikacje poświęcone projektom Wiesława Leśniewskiego i Stanisława Lejkowskiego</t>
+  </si>
+  <si>
+    <t>muszelkowe profilowane oparcie; jednolita tapicerowana skorupa; zaokrąglona górna krawędź oparcia; płynne przejście oparcia w siedzisko; brak podłokietników; cztery smukłe stożkowe drewniane nogi; lekka organiczna bryła; profilowana skorupa ze sklejki; niewielki prześwit pod siedziskiem; forma inspirowana muszlą</t>
+  </si>
+  <si>
+    <t>Bumerang</t>
+  </si>
+  <si>
+    <t>Ryszard Kulm</t>
+  </si>
+  <si>
+    <t>przełom lat 50. i 60. XX w.; produkcja seryjna od początku lat 60</t>
+  </si>
+  <si>
+    <t>Gościcińska Fabryka Mebli</t>
+  </si>
+  <si>
+    <t>charakterystyczne łukowato wygięte przednie nogi przypominające bumerang; lekka ażurowa konstrukcja; tapicerowane siedzisko; tapicerowane oparcie; smukła sylwetka; zwężające się ku dołowi nogi; modernistyczna forma inspirowana skandynawskim wzornictwem</t>
+  </si>
+  <si>
+    <t>drewniany stelaż bukowy; gięte elementy boczne; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; połączenia skręcane i klejone</t>
+  </si>
+  <si>
+    <t>GFM-22; typ 200-190 Rajmunda Hałasa; GFM-57 Skoczek; krzesła skandynawskie lat 60</t>
+  </si>
+  <si>
+    <t>krzesła Gościcińskiej Fabryki Mebli; wariant 299XB (Do weryfikacji); rodzina krzeseł Bumerang</t>
+  </si>
+  <si>
+    <t>Meblostan – Komplet 4 krzeseł Bumerang typ 299; Skarby PRL – Krzesło tapicerowane Bumerang typ 299; Patyna – Komplet krzeseł typ 299 Bumerang; Deccoria – 10 słynnych mebli z PRL; Stary Fotel – Krzesła Bumerang metamorfoza</t>
+  </si>
+  <si>
+    <t>łukowato wygięte przednie nogi w kształcie bumerangu; gięte boczne elementy drewniane; tapicerowane prostokątne siedzisko; tapicerowane oparcie; smukła lekka bryła; cienki drewniany stelaż; zwężające się ku dołowi nogi; wyraźny prześwit pod siedziskiem; organiczny profil boczny; lekko odchylone oparcie; minimalistyczna forma lat 60.; charakterystyczna sylwetka bumerangu</t>
+  </si>
+  <si>
+    <t>Typ 300-227</t>
+  </si>
+  <si>
+    <t>Celia</t>
+  </si>
+  <si>
+    <t>ok. 1965; produkcja na przełomie lat 60. i 70. XX w.</t>
+  </si>
+  <si>
+    <t>Zamojskie Fabryki Mebli</t>
+  </si>
+  <si>
+    <t>brak podłokietników; toczone drewniane nogi umieszczone po bokach części tapicerowanej; trapezowe siedzisko; proste tapicerowane oparcie; lekka minimalistyczna forma; kompaktowe wymiary; stylistyka skandynawskiego modernizmu</t>
+  </si>
+  <si>
+    <t>drewniany stelaż; toczone nogi; tapicerowane siedzisko; tapicerowane oparcie; otwarta konstrukcja bez podłokietników; konstrukcja szkieletowa przeznaczona do produkcji seryjnej</t>
+  </si>
+  <si>
+    <t>typ 300-190 Lisek; typ 366; GFM-64; lekkie fotele klubowe PRL bez podłokietników</t>
+  </si>
+  <si>
+    <t>fotele Zamojskich Fabryk Mebli z lat 60. i 70.; meble klubowe produkowane w Zamościu; modele o minimalistycznej konstrukcji bez podłokietników</t>
+  </si>
+  <si>
+    <t>Meblostan – Fotel CELIA typ 300-227; Patyna – Fotel CELIA typ 300-227 PRL; Szajba Sklep – Fotel Celia typ 300-227; materiały kolekcjonerskie dotyczące Zamojskich Fabryk Mebli</t>
+  </si>
+  <si>
+    <t>brak podłokietników; toczone drewniane nogi umieszczone po bokach korpusu; trapezowe tapicerowane siedzisko; prostokątne tapicerowane oparcie; lekka minimalistyczna bryła; duży prześwit pod siedziskiem; cienki drewniany stelaż; zwężające się ku dołowi nogi; odsłonięte drewniane elementy boczne; kompaktowe proporcje; geometryczny profil boczny; forma inspirowana skandynawskim modernizmem</t>
+  </si>
+  <si>
+    <t>Typ 300-139</t>
+  </si>
+  <si>
+    <t>Stefan</t>
+  </si>
+  <si>
+    <t>Swarzędzka Fabryka Mebli</t>
+  </si>
+  <si>
+    <t>szerokie drewniane podłokietniki o łagodnym łuku; otwarta konstrukcja boczna; luźne tapicerowane poduchy siedziska i oparcia; rozłożysta bryła; lekka skandynawska stylistyka; nisko osadzone siedzisko; masywny drewniany stelaż</t>
+  </si>
+  <si>
+    <t>stelaż z litego drewna bukowego; otwarta rama boczna; osobna poduszka siedziska; osobna poduszka oparcia; pasy tapicerskie; konstrukcja szkieletowa skręcana</t>
+  </si>
+  <si>
+    <t>typ 300-123 Puchała; typ 366; duńskie fotele Kandidaten projektu Ib Kofod-Larsena; fotele skandynawskie lat 60</t>
+  </si>
+  <si>
+    <t>sofa Stefan; zestawy wypoczynkowe Swarzędzkiej Fabryki Mebli; meble eksportowe Swarzędzkiej Fabryki Mebli z lat 60.</t>
+  </si>
+  <si>
+    <t>„Meble w produkcji 1962” – Zjednoczenie Przemysłu Meblarskiego; „Meble do małych mieszkań. Informator”, Wydawnictwo Katalogów i Cenników 1966; Laminerva – „Ikony polskiego designu: Fotel Stefan typ 300-139”; Meblostan – Para foteli Stefan typ 300-139; Patyna – Para foteli Stefan typ 300-139</t>
+  </si>
+  <si>
+    <t>szerokie wyprofilowane drewniane podłokietniki; otwarta drewniana rama boczna; luźna poduszka siedziska; luźna poduszka oparcia; nisko osadzone głębokie siedzisko; prostokątne grube poduchy; lekko odchylone oparcie; masywny bukowy stelaż; duży prześwit pod siedziskiem; szeroki rozstaw przednich nóg; profil boczny inspirowany wzornictwem skandynawskim; rozłożysta bryła eksportowa</t>
+  </si>
+  <si>
+    <t>B-3300</t>
+  </si>
+  <si>
+    <t>ok. 1969; produkcja w końcu lat 60. i na początku lat 70. XX w</t>
+  </si>
+  <si>
+    <t>Zakład Mebli Giętych w Radomsku; Fabryki Mebli Radomsko (późniejsze nazewnictwo zakładu)</t>
+  </si>
+  <si>
+    <t>gięte drewniane podłokietniki; szerokie tapicerowane siedzisko; prostokątne tapicerowane oparcie; otwarta konstrukcja boczna; gięty bukowy stelaż; nisko osadzona bryła; elegancka modernistyczna forma</t>
+  </si>
+  <si>
+    <t>stelaż z giętego drewna bukowego; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; elementy gięte wykonane w technologii Thoneta; konstrukcja skręcana</t>
+  </si>
+  <si>
+    <t>B-310 VAR; B-6028; GFM-64; typ 300-139 Stefan</t>
+  </si>
+  <si>
+    <t>fotele Zakładu Mebli Giętych w Radomsku; modele eksportowe Radomsko z lat 60. i 70.; rodzina foteli z giętego drewna bukowego</t>
+  </si>
+  <si>
+    <t>Patyna – Fotel B-3300 Zakład Mebli Giętych w Radomsku; Meblostan – Para foteli B-3300; archiwalne materiały Fabryk Mebli Radomsko; oferty kolekcjonerskie dokumentujące oryginalne oznaczenie modelu</t>
+  </si>
+  <si>
+    <t>gięte drewniane podłokietniki; otwarta drewniana rama boczna; szerokie prostokątne oparcie; szerokie głębokie siedzisko; bukowy gięty stelaż; duży prześwit pod siedziskiem; łagodnie wygięte boki; zwężające się ku dołowi nogi; lekko pochylone oparcie; masywniejsza bryła niż typ 366; widoczne elementy z giętego drewna; modernistyczna forma gabinetowa</t>
+  </si>
+  <si>
+    <t>Cechy AI</t>
   </si>
   <si>
     <t>drewniane boczki;
@@ -382,33 +1057,6 @@
 brak ozdobnych detali</t>
   </si>
   <si>
-    <t>Fotel typ 300-190</t>
-  </si>
-  <si>
-    <t>Lisek</t>
-  </si>
-  <si>
-    <t>Henryk Lis</t>
-  </si>
-  <si>
-    <t>Dolnośląska Fabryka Mebli w Świebodzicach; Bystrzyckie Fabryki Mebli; Zakład Mebli Giętych FAMEG Radomsko; Świdnicki Ośrodek Przemysłu Meblarskiego</t>
-  </si>
-  <si>
-    <t>Fotel posiada lekką, smukłą konstrukcję opartą na odsłoniętej drewnianej ramie. Tapicerowane siedzisko i oparcie osadzone są pomiędzy drewnianymi boczkami zakończonymi płaskimi podłokietnikami. Konstrukcja wsparta jest na czterech toczonych, lekko zwężających się nogach. W połowie wysokości nóg widoczne są poprzeczne belki tworzące charakterystyczną ramę usztywniającą. Drewniane elementy wykończone były lakierem o wykończeniu matowym, półmatowym lub z połyskiem.</t>
-  </si>
-  <si>
-    <t>Konstrukcję nośną tworzą drewniane boczki połączone poprzecznymi belkami oraz stelażem. Nogi są mocowane do płaskich podłokietników. Do wykonania stolarki zastosowano drewno bukowe. Siedzisko wykorzystuje formatki gumowe osadzone na elastycznych pasach zamiast sprężyn i tradycyjnych wypełnień.</t>
-  </si>
-  <si>
-    <t>typ 366; GFM-64; fotele klubowe PRL z lat 60.</t>
-  </si>
-  <si>
-    <t>zestaw Odra; zestaw Syrena; warianty produkcyjne różnych fabryk (Do weryfikacji)</t>
-  </si>
-  <si>
-    <t>Nowohuckie Renowacje – Fotel Lisek typ 300-190; Conchita Home – 4 fotele z PRL które musisz znać; dokumentacja i opisy egzemplarzy Typ 300-190; archiwalne materiały producentów cytowane w opracowaniach specjalistycznych</t>
-  </si>
-  <si>
     <t>toczone nogi;
 lekko zwężające się nogi;
 cztery drewniane nogi;
@@ -436,33 +1084,6 @@
 minimalistyczna forma</t>
   </si>
   <si>
-    <t>Do weryfikacji; często błędnie określany jako „Lisek”</t>
-  </si>
-  <si>
-    <t>Henryk Lis (do potwierdzenia)</t>
-  </si>
-  <si>
-    <t>1969–1970</t>
-  </si>
-  <si>
-    <t>Zakłady Przemysłu Meblarskiego im. Gwardii Ludowej w Radomsku; Fabryki Mebli Radomsko</t>
-  </si>
-  <si>
-    <t>Fotel posiada otwartą drewnianą konstrukcję zewnętrzną wykonaną z litego drewna. Tapicerowane siedzisko i oparcie zamocowane są wewnątrz drewnianej ramy za pomocą wkrętów lub śrub. Konstrukcja opiera się na czterech toczonych nogach połączonych belkami podtrzymującymi siedzisko. Charakterystycznym elementem są zaokrąglone drewniane podłokietniki stanowiące integralną część bocznej ramy.</t>
-  </si>
-  <si>
-    <t>Konstrukcja wykonana jest z litej tarcicy bukowej. Szkielet ukryty pod tapicerką wykonano z tarcicy iglastej. Siedzisko i oparcie mocowane są do ramy za pomocą wkrętów lub śrub. Połączenia konstrukcyjne obejmują połączenia czopowe oraz połączenia na wkręty. W siedzisku zastosowano pasy tapicerskie i tworzywo piankowe.</t>
-  </si>
-  <si>
-    <t>typ 300-190 Lisek; BW-14; typ 366</t>
-  </si>
-  <si>
-    <t>rodzina foteli Radomsko o otwartej konstrukcji ramowej; BW-14; typ 300-190 Lisek (wizualnie pokrewny)</t>
-  </si>
-  <si>
-    <t>Patyna.pl – fotel B-7727 Radomsko PRL; Meblostan – fotel B-7727; Nowohuckie Renowacje – fotel B-7727; Vilandy – fotel Lis typ B-7727; Allegro – fotel PRL model B-7727 Radomsko lata 70; Reko-Czyny – identyfikacja fotela B-7727</t>
-  </si>
-  <si>
     <t>toczone nogi;
 cztery drewniane nogi;
 zaokrąglone podłokietniki;
@@ -487,63 +1108,6 @@
 widoczne mocowanie siedziska;
 widoczne mocowanie oparcia;
 drewniany stelaż</t>
-  </si>
-  <si>
-    <t>Typ 300-177</t>
-  </si>
-  <si>
-    <t>Bunny; Zajączek</t>
-  </si>
-  <si>
-    <t>Józef Chierowski (Do weryfikacji – atrybucja często powtarzana w źródłach kolekcjonerskich, słabo potwierdzona w publikacjach naukowych)</t>
-  </si>
-  <si>
-    <t>początek lat 60. XX w.</t>
-  </si>
-  <si>
-    <t>Świebodzińskie Fabryki Mebli; Gościcińskie Fabryki Mebli</t>
-  </si>
-  <si>
-    <t>trójkątne podłokietniki; lekka drewniana konstrukcja; kompaktowe wymiary; szeroko rozstawione nogi; tapicerowane siedzisko i oparcie; forma nawiązująca do modelu 366</t>
-  </si>
-  <si>
-    <t>bukowy stelaż; otwarta konstrukcja boczna; tapicerowane moduły siedziska i oparcia; drewniane podłokietniki zintegrowane z ramą; konstrukcja szkieletowa</t>
-  </si>
-  <si>
-    <t>typ 366; typ 300-190 Lisek; BW-14</t>
-  </si>
-  <si>
-    <t>typ 366; grupa lekkich foteli drewnianych PRL z lat 60.; modele produkowane przez Świebodzińskie i Gościcińskie Fabryki Mebli (Do weryfikacji)</t>
-  </si>
-  <si>
-    <t>Meblostan – Fotel Bunny typ 300-177; Nowohuckie Renowacje – Fotel typ 300-177 Zajączek; Patyna.pl – Fotel Bunny typ 300-177; Tkaniny-Meblowe.pl – Fotele z PRL-u; materiały kolekcjonerskie rynku vintage</t>
-  </si>
-  <si>
-    <t>trójkątne podłokietniki przypominające uszy zająca; otwarta drewniana rama boczna; szeroko rozstawione nogi; podłokietniki połączone z przednimi nogami; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; smukła lekka bryła; odsłonięty drewniany stelaż; skośne tylne nogi; geometryczny profil boczny; kompaktowe proporcje</t>
-  </si>
-  <si>
-    <t>Fotel Ewa; Muszelka Ewa</t>
-  </si>
-  <si>
-    <t>Do weryfikacji</t>
-  </si>
-  <si>
-    <t>Strzeleckie Zakłady Przemysłu Terenowego w Strzelcach Opolskich</t>
-  </si>
-  <si>
-    <t>Fotel posiada muszelkowy, kubełkowy korpus tworzący jednolitą tapicerowaną bryłę. Szerokie, półkoliste oparcie płynnie przechodzi w siedzisko, nadając bryle profil przypominający muszlę. Korpus osadzony jest na odsłoniętym stalowym stelażu wspartym na czterech smukłych metalowych nogach. Fotel nie posiada drewnianych podłokietników, a wysoka podstawa nadaje konstrukcji lekką formę.</t>
-  </si>
-  <si>
-    <t>Konstrukcję nośną stanowi rama wykonana ze spawanych prętów stalowych. Rama wsparta jest na czterech stalowych, wykręcanych nogach zakończonych ruchomymi stopkami. W modelu Koeln 1 zastosowano pojedynczą stalową nogę obrotową.</t>
-  </si>
-  <si>
-    <t>fotel Köln 1; fotel Muszelka; fotele klubowe na stelażu stalowym z lat 60.</t>
-  </si>
-  <si>
-    <t>Köln 1 (NRD); fotele muszelkowe PRL; metalowe fotele klubowe lat 60.</t>
-  </si>
-  <si>
-    <t>Meblostan – Para foteli tapicerowanych EWA; Odnowa Mebli – Fotel Ewa; Patyna.pl – Komplet foteli typ Ewa; materiały kolekcjonerskie rynku vintage</t>
   </si>
   <si>
     <t>muszelkowy korpus;
@@ -571,458 +1135,6 @@
 otwarta konstrukcja;
 obszerne siedzisko;
 obszerne oparcie</t>
-  </si>
-  <si>
-    <t>Typ 300-123</t>
-  </si>
-  <si>
-    <t>Puchała; wersja damska (Do weryfikacji)</t>
-  </si>
-  <si>
-    <t>Mieczysław Puchała</t>
-  </si>
-  <si>
-    <t>1956 (według części źródeł); początek lat 60. XX w.</t>
-  </si>
-  <si>
-    <t>lekka smukła sylwetka; gięte drewniane podłokietniki; wysokie oparcie; wąskie proporcje; odsłonięta drewniana konstrukcja; toczone nogi; modernistyczna forma inspirowana wzornictwem skandynawskim</t>
-  </si>
-  <si>
-    <t>drewniany stelaż bukowy; otwarta konstrukcja boczna; tapicerowane siedzisko; tapicerowane oparcie; pasy tapicerskie; konstrukcja szkieletowa</t>
-  </si>
-  <si>
-    <t>typ 300-137; typ 300-190 Lisek; typ 366</t>
-  </si>
-  <si>
-    <t>typ 300-137 wersja męska; rodzina foteli projektu Mieczysława Puchały; lekkie fotele drewniane PRL lat 50. i 60</t>
-  </si>
-  <si>
-    <t>Nowohuckie Renowacje – Fotel typ 300-123 Puchała; Szajba Sklep – Fotel klubowy typ 300-123 proj. M. Puchała; LookInside – Fotel typ 300-123 Puchała; Pakamera – Fotel typ 300-123 M. Puchała; Meblostan – Fotel Puchały typ 300-123</t>
-  </si>
-  <si>
-    <t>gięte drewniane podłokietniki; smukłe wysokie oparcie; wąskie proporcje korpusu; otwarta drewniana rama boczna; toczone nogi zwężające się ku dołowi; widoczny prześwit pod siedziskiem; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; lekka dynamiczna bryła; cienkie elementy konstrukcyjne; profil boczny z łukowato wygiętym podłokietnikiem; minimalistyczna forma lat 50./60.</t>
-  </si>
-  <si>
-    <t>RM58</t>
-  </si>
-  <si>
-    <t>Muszelka; RM58</t>
-  </si>
-  <si>
-    <t>Roman Modzelewski</t>
-  </si>
-  <si>
-    <t>Zakłady Mebli Artystycznych w Łodzi (prototyp); Vzór Sp. z o.o. (reedycja od 2012 r.)</t>
-  </si>
-  <si>
-    <t>organiczna muszelkowa forma; jednolita zamknięta bryła; głębokie kubełkowe siedzisko; szerokie wywinięte boki; opływowy futurystyczny kształt; brak klasycznych podłokietników; rzeźbiarska sylwetka</t>
-  </si>
-  <si>
-    <t>jednoczęściowy korpus z laminatu poliestrowo-szklanego; tapicerowana wkładka siedziska; cztery smukłe nogi; technologia laminatu wyprzedzająca epokę w Polsce; konstrukcja skorupowa</t>
-  </si>
-  <si>
-    <t>fotel Ewa; fotele muszelkowe produkcji NRD; zachodnie fotele fiberglass lat 50.; projekty Eero Saarinena</t>
-  </si>
-  <si>
-    <t>prototypowe meble z laminatu Romana Modzelewskiego; współczesne reedycje RM58; warianty kolorystyczne RM58 Classic</t>
-  </si>
-  <si>
-    <t>Muzeum Narodowe we Wrocławiu; Vzór – dokumentacja reedycji RM58; Instytut Wzornictwa Przemysłowego; publikacje o twórczości Romana Modzelewskiego; Culture.pl</t>
-  </si>
-  <si>
-    <t>jednoczęściowa muszelkowa skorupa; organiczna opływowa bryła; głębokie kubełkowe siedzisko; szerokie wywinięte boki; zaokrąglone wysokie oparcie; brak oddzielnych podłokietników; korpus przypominający muszlę; zamknięta forma boczna; cztery cienkie nogi; futurystyczna sylwetka lat 50.; brak widocznej drewnianej konstrukcji; płynne przejścia między siedziskiem i oparciem; asymetrycznie zaokrąglone krawędzie; korpus wykonany jako pojedyncza skorupa</t>
-  </si>
-  <si>
-    <t>B-2020</t>
-  </si>
-  <si>
-    <t>Tulipan</t>
-  </si>
-  <si>
-    <t>Teresa Kruszewska</t>
-  </si>
-  <si>
-    <t>1973 (prototyp)</t>
-  </si>
-  <si>
-    <t>FAMEG Radomsko (reedycja współczesna)</t>
-  </si>
-  <si>
-    <t>organiczna forma inspirowana kielichem kwiatu; szerokie kubełkowe siedzisko; płynne przejście między siedziskiem i oparciem; miękkie zaokrąglone linie; wyraźnie rozchylone boki; rzeźbiarska bryła</t>
-  </si>
-  <si>
-    <t>korpus ze sklejki formowanej; tapicerowana skorupa; drewniana podstawa; konstrukcja monolityczna; technologia giętej sklejki</t>
-  </si>
-  <si>
-    <t>RM58; fotele muszelkowe PRL; fotele skandynawskie o organicznej formie</t>
-  </si>
-  <si>
-    <t>projekty Teresy Kruszewskiej; meble ze sklejki formowanej; współczesna kolekcja Tulipan FAMEG</t>
-  </si>
-  <si>
-    <t>FAMEG – Fotel Tulipan B-2020; dokumentacja reedycji FAMEG; opracowania dotyczące twórczości Teresy Kruszewskiej</t>
-  </si>
-  <si>
-    <t>kubełkowe siedzisko; forma przypominająca kielich tulipana; szeroko rozchylone boki; jednolita tapicerowana skorupa; zaokrąglone wysokie oparcie; płynne przejście między siedziskiem i oparciem; organiczna bryła; brak widocznej drewnianej ramy bocznej; miękkie obłe krawędzie; rzeźbiarska forma; kompaktowa podstawa; sylwetka kwiatu tulipana</t>
-  </si>
-  <si>
-    <t>Typ 300-201</t>
-  </si>
-  <si>
-    <t>Śnieżnik; Śnieżka (Do weryfikacji – obie nazwy występują w obiegu kolekcjonerskim, częściej spotykana jest nazwa Śnieżnik)</t>
-  </si>
-  <si>
-    <t>1973 (najwcześniejsza potwierdzona wzmianka źródłowa)</t>
-  </si>
-  <si>
-    <t>Bystrzycka Fabryka Mebli w Bystrzycy Kłodzkiej</t>
-  </si>
-  <si>
-    <t>lekka konstrukcja drewniana; forma inspirowana modelem Lisek 300-190; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; otwarta rama boczna; charakterystyczne nogi częściowo graniaste i częściowo zaokrąglone; smukłe proporcje</t>
-  </si>
-  <si>
-    <t>drewniany stelaż brzozowy lub bukowy; otwarta konstrukcja boczna; tapicerowane siedzisko; tapicerowane oparcie; pasy tapicerskie; konstrukcja szkieletowa</t>
-  </si>
-  <si>
-    <t>typ 300-190 Lisek; Śnieżka; BW-14 typ 300-199; B-7727</t>
-  </si>
-  <si>
-    <t>typ 300-190 Lisek; Śnieżka; BW-14 typ 300-199; BW-20 typ 300-193; B-7727</t>
-  </si>
-  <si>
-    <t>Meblostan – Fotel Śnieżnik typ 300-201; Nowohuckie Renowacje – Fotele PRL; Pakamera – Fotel Śnieżnik typ 300-201; Audiovintage Store – Fotel klubowy Śnieżnik 300-201</t>
-  </si>
-  <si>
-    <t>otwarta drewniana rama boczna; prostokątne tapicerowane oparcie; prostokątne tapicerowane siedzisko; smukła lekka bryła; duży prześwit pod siedziskiem; drewniane podłokietniki zintegrowane z ramą; nogi graniaste od góry; nogi zaokrąglone w dolnej części; skośne tylne nogi; widoczne drewniane elementy konstrukcyjne; forma zbliżona do modelu Lisek; geometryczny profil boczny
-Źródła potwierdzają produkcję w Bystrzyckiej Fabryce Mebli oraz silne pokrewieństwo konstrukcyjne z modelem 300-190 „Lisek”, natomiast projektant pozostaje niepotwierdzony.</t>
-  </si>
-  <si>
-    <t>GFM-57</t>
-  </si>
-  <si>
-    <t>Skoczek</t>
-  </si>
-  <si>
-    <t>Juliusz Kędziorek</t>
-  </si>
-  <si>
-    <t>Krzesło</t>
-  </si>
-  <si>
-    <t>Gościcińska Fabryka Mebli; Zamojskie Fabryki Mebli (produkcja seryjna jako typ 200-203)</t>
-  </si>
-  <si>
-    <t>łukowate podłokietniki przypominające profil skoczni narciarskiej; elipsoidalne oparcie; lekka ażurowa konstrukcja; zwężające się ku dołowi nogi; tapicerowane siedzisko; smukła sylwetka; organiczna linia boczna</t>
-  </si>
-  <si>
-    <t>drewniany stelaż; otwarta konstrukcja boczna; tapicerowane siedzisko; gięte elementy drewniane; konstrukcja przeznaczona do produkcji seryjnej</t>
-  </si>
-  <si>
-    <t>typ 200-190 Rajmunda Hałasa; krzesła Aga; krzesła patyczaki lat 60.; lekkie krzesła tapicerowane PRL</t>
-  </si>
-  <si>
-    <t>typ 200-203; GFM-107; projekty Juliusza Kędziorka dla Gościcińskiej Fabryki Mebli</t>
-  </si>
-  <si>
-    <t>Magazif – Krzesło Skoczek; Ikony Designu PL – Krzesło GFM-57 Skoczek; Meblostan – Krzesło Skoczek; Sosenko Home Decor – Krzesło Skoczek; Allegro Artykuł – Krzesło kilka słów o najtrudniejszym meblu</t>
-  </si>
-  <si>
-    <t>łukowate podłokietniki przypominające skocznię narciarską; elipsoidalne oparcie; otwarta drewniana rama boczna; smukłe zwężające się nogi; tapicerowane siedzisko; duży prześwit pod siedziskiem; płynna linia podłokietnika przechodząca w nogę; lekka ażurowa konstrukcja; organiczny profil boczny; oparcie w kształcie pionowej elipsy; cienkie elementy drewniane; dynamiczna sylwetka inspirowana skokami narciarskimi
-Źródła potwierdzają, że model został zaprojektowany przez Juliusza Kędziorka w Gościcińskiej Fabryce Mebli w 1965 r., otrzymał nagrodę „Dobre–Ładne–Poszukiwane” i został skierowany do produkcji seryjnej jako typ 200-203</t>
-  </si>
-  <si>
-    <t>Typ 200-125 VAR</t>
-  </si>
-  <si>
-    <t>Aga</t>
-  </si>
-  <si>
-    <t>ok. 1972–1975 (w źródłach występują rozbieżności dotyczące dokładnego roku projektu)</t>
-  </si>
-  <si>
-    <t>Wielkopolskie Fabryki Mebli; produkcja seryjna PRL (pozostali producenci wymagają weryfikacji)</t>
-  </si>
-  <si>
-    <t>wysokie tapicerowane oparcie; trapezowy układ nóg; miękkie tapicerowane siedzisko; smukła skandynawska forma; zwężająca się ku górze bryła; lekkie proporcje; drewniana konstrukcja eksponowana po bokach</t>
-  </si>
-  <si>
-    <t>drewniany stelaż bukowy; tapicerowane siedzisko; tapicerowane oparcie; sprężyny siedziska; cztery drewniane nogi; konstrukcja przeznaczona do intensywnego użytkowania klubowego</t>
-  </si>
-  <si>
-    <t>typ 200-190 Rajmunda Hałasa; GFM-57 Skoczek; lekkie krzesła klubowe PRL lat 70.</t>
-  </si>
-  <si>
-    <t>fotel 366; meble klubowe Józefa Chierowskiego; reedycja 200-125 VAR realizowana przez 366 Concept</t>
-  </si>
-  <si>
-    <t>Elle Decoration Polska – Krzesło VAR AGA projektu Józefa Chierowskiego; Nowohuckie Renowacje – Krzesło Aga typ 200-125; Patyna.pl – Krzesła AGA typu 200-125 VAR; Linie Studio – 200-125 VAR; Meblościanka – 200-125 VAR</t>
-  </si>
-  <si>
-    <t>wysokie tapicerowane oparcie; trapezowy układ nóg; szerokie miękkie siedzisko; brak podłokietników; drewniane nogi rozszerzające się ku dołowi; zwężająca się ku górze sylwetka; lekka skandynawska forma; prostokątne oparcie z zaokrąglonymi krawędziami; widoczne drewniane elementy boczne; smukłe proporcje; geometryczna bryła; profil boczny z pochylonym oparciem</t>
-  </si>
-  <si>
-    <t>Typ 200-190</t>
-  </si>
-  <si>
-    <t>Hałas; Grzybek</t>
-  </si>
-  <si>
-    <t>Rajmund Teofil Hałas</t>
-  </si>
-  <si>
-    <t>lata 60. XX w.; dokładny rok projektu – Do weryfikacji</t>
-  </si>
-  <si>
-    <t>Zakłady Mebli w Gostyniu (Do weryfikacji); produkcja seryjna w kilku zakładach meblarskich PRL – Do weryfikacji</t>
-  </si>
-  <si>
-    <t>okrągła forma oparcia przypominająca kapelusz grzyba; tapicerowane oparcie i siedzisko; smukłe zwężające się nogi; lekka konstrukcja; wyraźnie wyodrębnione oparcie nad siedziskiem; proporcje inspirowane wzornictwem skandynawskim; minimalistyczna sylwetka</t>
-  </si>
-  <si>
-    <t>drewniany stelaż; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; mocowane oddzielnie siedzisko i oparcie; nogi zwężające się ku dołowi</t>
-  </si>
-  <si>
-    <t>Aga 200-125; Skoczek GFM-57; krzesła skandynawskie lat 60.; lekkie krzesła tapicerowane PRL</t>
-  </si>
-  <si>
-    <t>projekty Rajmunda Teofila Hałasa; krzesła tapicerowane PRL lat 60.; warianty produkcyjne typu 200-190</t>
-  </si>
-  <si>
-    <t>Odnawialnia – Wiem co odnawiam | krzesło Hałasa typ 200-190; Patyna.pl – Krzesła typ 200-190 Rajmund Teofil Hałas; Meblostan – Komplet krzeseł typ 200-190; Daniel Stoiński Redesign – Przewodnik po renowacji krzesła 200-190; Homebook – Krzesło Hałasa typ 200-190</t>
-  </si>
-  <si>
-    <t>okrągłe oparcie przypominające grzybek; oparcie szersze od wspornika; tapicerowane okrągłe oparcie; tapicerowane siedzisko; smukłe nogi zwężające się ku dołowi; brak podłokietników; lekka skandynawska forma; duży prześwit pod siedziskiem; cienki drewniany stelaż; wyraźne oddzielenie oparcia od siedziska; geometryczna bryła; profil boczny z lekko odchylonym oparciem</t>
-  </si>
-  <si>
-    <t>B-6028</t>
-  </si>
-  <si>
-    <t>Barbara Fenrych-Węcławska (Do weryfikacji); Józef Chierowski (Do weryfikacji – atrybucja pojawiająca się wyłącznie w źródłach kolekcjonerskich)</t>
-  </si>
-  <si>
-    <t>lata 60. XX w.</t>
-  </si>
-  <si>
-    <t>Fabryka Mebli Giętych w Radomsku; FAMEG Radomsko; Radomszczańska Fabryka Mebli Giętych</t>
-  </si>
-  <si>
-    <t>wysokie profilowane oparcie; szerokie drewniane podłokietniki; gięte elementy bukowe; głębokie siedzisko; lekka otwarta konstrukcja boczna; elegancka smukła sylwetka; forma łącząca cechy fotela klubowego i wypoczynkowego</t>
-  </si>
-  <si>
-    <t>stelaż z giętego drewna bukowego; otwarta konstrukcja ramowa; tapicerowane siedzisko; tapicerowane oparcie; drewniane podłokietniki zintegrowane z ramą; konstrukcja szkieletowa</t>
-  </si>
-  <si>
-    <t>typ 300-123 Puchała; typ 300-177 Zajączek; B-7727; typ 366</t>
-  </si>
-  <si>
-    <t>fotele Radomsko z giętego drewna; projekty Barbary Fenrych-Węcławskiej (Do weryfikacji); lekkie fotele klubowe PRL lat 60.</t>
-  </si>
-  <si>
-    <t>MidMod – Fotel B6028 FAMEG Radomsko Polska lata 60; Oldsen Design – Fotel B6028 prod. FAMEG Radomsko; Nowohuckie Renowacje – Fotel PRL B-6028 z lat 60-tych; Fotelowo Facebook – fotel projektu Barbary Fenrych-Węcławskiej; Instagram Renowacja Mebli PRL – B6028 lata produkcji 1960</t>
-  </si>
-  <si>
-    <t>wysokie prostokątne oparcie; szerokie drewniane podłokietniki; gięte boczne elementy z drewna; otwarta rama boczna; głębokie siedzisko; masywniejsza bryła niż typ 366; bukowy stelaż; duży prześwit pod siedziskiem; profilowane podłokietniki; smukłe nogi zintegrowane z ramą; tapicerowane oparcie i siedzisko; geometryczny profil boczny</t>
-  </si>
-  <si>
-    <t>A. Dutka</t>
-  </si>
-  <si>
-    <t>1966–1968</t>
-  </si>
-  <si>
-    <t>Zakłady Mebli Giętych w Radomsku; Gołuchowskie Fabryki Mebli</t>
-  </si>
-  <si>
-    <t>duże gabaryty; szerokie głębokie siedzisko; masywne drewniane podłokietniki; geometryczna forma boczna; lekko pochylone oparcie; otwarta konstrukcja ramowa; modernistyczna sylwetka eksportowa</t>
-  </si>
-  <si>
-    <t>stelaż z drewna bukowego; sprężyny lejowe w siedzisku; tapicerowane siedzisko i oparcie; otwarta konstrukcja boczna; drewniane podłokietniki zintegrowane z ramą; konstrukcja rozbieralna skręcana śrubami</t>
-  </si>
-  <si>
-    <t>B-6028; GFM-64; typ 300-190 Lisek; B-7727</t>
-  </si>
-  <si>
-    <t>fotele eksportowe Radomsko lat 60.; modele Zakładów Mebli Giętych w Radomsku; konstrukcje projektowane przez A. Dutkę (Do weryfikacji)</t>
-  </si>
-  <si>
-    <t>Meblostan – Para foteli B-310 VAR; Pufa Design – Oryginalny fotel B-310 VAR; Yestersen – Fotel B-310 VAR Polska lata 70.; Reko-Czyny – Fotel B-310 VAR metamorfoza; archiwalne ogłoszenia kolekcjonerskie B-310 VAR</t>
-  </si>
-  <si>
-    <t>masywne drewniane podłokietniki; szerokie głębokie siedzisko; wysunięte przednie podłokietniki; otwarta drewniana rama boczna; prostokątne tapicerowane oparcie; grube proporcje siedziska; lekko pochylone oparcie; duży prześwit pod siedziskiem; widoczne śruby montażowe w ramie; geometryczny profil boczny; szeroki rozstaw nóg; cięższa bryła niż typ 366; bukowy stelaż; modernistyczna forma eksportowa</t>
-  </si>
-  <si>
-    <t>GFM-22 (typ 200/128)</t>
-  </si>
-  <si>
-    <t>ok. 1960</t>
-  </si>
-  <si>
-    <t>Gościcińska Fabryka Mebli (GFM)</t>
-  </si>
-  <si>
-    <t>nerkowate oparcie; lekka ażurowa konstrukcja; smukłe zwężające się nogi; gięta drewniana rama; tapicerowane siedzisko; tapicerowane oparcie; wyraźnie rozstawione tylne nogi</t>
-  </si>
-  <si>
-    <t>drewniany stelaż; gięte elementy z litego drewna; tapicerowane siedzisko; tapicerowane oparcie ze sklejki giętej; konstrukcja szkieletowa przeznaczona do produkcji seryjnej</t>
-  </si>
-  <si>
-    <t>GFM-57 Skoczek; typ 200-190 Rajmunda Hałasa; Aga 200-125; krzesła skandynawskie z lat 60.</t>
-  </si>
-  <si>
-    <t>typ 200/128; projekty Juliusza Kędziorka dla Gościcińskiej Fabryki Mebli; GFM-57; GFM-87</t>
-  </si>
-  <si>
-    <t>Pamono – Mid-Century GFM-22 Chairs by Juliusz Kędziorek; Vinterior – GFM-22 model 200/128; Selency – Iconic GFM-22 Chair by Juliusz Kędziorek; Instagram Zostań z Vintage – Krzesło GFM-22 typ 200/128</t>
-  </si>
-  <si>
-    <t>nerkowate tapicerowane oparcie; oparcie szersze od wspornika; smukłe zwężające się nogi; lekka ażurowa konstrukcja; gięta drewniana rama; prostokątne tapicerowane siedzisko; duży prześwit pod siedziskiem; cienkie elementy konstrukcyjne; szeroko rozstawione tylne nogi; profil boczny z delikatnie pochylonym oparciem; organiczny kształt oparcia; minimalistyczna sylwetka lat 60.</t>
-  </si>
-  <si>
-    <t>Typ 1020</t>
-  </si>
-  <si>
-    <t>Muszelka</t>
-  </si>
-  <si>
-    <t>Wiesław Leśniewski; Stanisław Lejkowski</t>
-  </si>
-  <si>
-    <t>Słupskie Fabryki Mebli</t>
-  </si>
-  <si>
-    <t>muszelkowe profilowane oparcie; jednolita tapicerowana skorupa; zaokrąglona górna krawędź oparcia; smukłe stożkowe nogi; lekka modernistyczna forma; brak podłokietników; organiczna sylwetka</t>
-  </si>
-  <si>
-    <t>profilowana skorupa ze sklejki; tapicerowana skorupa; drewniany stelaż; cztery drewniane nogi; konstrukcja szkieletowa; połączenie sklejki i drewna litego</t>
-  </si>
-  <si>
-    <t>RM58; krzesła muszelkowe produkcji NRD; krzesła skandynawskie lat 60.; fotel Ewa</t>
-  </si>
-  <si>
-    <t>krzesła muszelkowe Słupskich Fabryk Mebli; projekty Wiesława Leśniewskiego i Stanisława Lejkowskiego; meble ze sklejki profilowanej produkowane przez SFM</t>
-  </si>
-  <si>
-    <t>Archiwalne katalogi Słupskich Fabryk Mebli; opracowania kolekcjonerskie dotyczące wzornictwa SFM; materiały renowatorów specjalizujących się w meblach PRL; publikacje poświęcone projektom Wiesława Leśniewskiego i Stanisława Lejkowskiego</t>
-  </si>
-  <si>
-    <t>muszelkowe profilowane oparcie; jednolita tapicerowana skorupa; zaokrąglona górna krawędź oparcia; płynne przejście oparcia w siedzisko; brak podłokietników; cztery smukłe stożkowe drewniane nogi; lekka organiczna bryła; profilowana skorupa ze sklejki; niewielki prześwit pod siedziskiem; forma inspirowana muszlą</t>
-  </si>
-  <si>
-    <t>Bumerang</t>
-  </si>
-  <si>
-    <t>Ryszard Kulm</t>
-  </si>
-  <si>
-    <t>przełom lat 50. i 60. XX w.; produkcja seryjna od początku lat 60</t>
-  </si>
-  <si>
-    <t>Gościcińska Fabryka Mebli</t>
-  </si>
-  <si>
-    <t>charakterystyczne łukowato wygięte przednie nogi przypominające bumerang; lekka ażurowa konstrukcja; tapicerowane siedzisko; tapicerowane oparcie; smukła sylwetka; zwężające się ku dołowi nogi; modernistyczna forma inspirowana skandynawskim wzornictwem</t>
-  </si>
-  <si>
-    <t>drewniany stelaż bukowy; gięte elementy boczne; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; połączenia skręcane i klejone</t>
-  </si>
-  <si>
-    <t>GFM-22; typ 200-190 Rajmunda Hałasa; GFM-57 Skoczek; krzesła skandynawskie lat 60</t>
-  </si>
-  <si>
-    <t>krzesła Gościcińskiej Fabryki Mebli; wariant 299XB (Do weryfikacji); rodzina krzeseł Bumerang</t>
-  </si>
-  <si>
-    <t>Meblostan – Komplet 4 krzeseł Bumerang typ 299; Skarby PRL – Krzesło tapicerowane Bumerang typ 299; Patyna – Komplet krzeseł typ 299 Bumerang; Deccoria – 10 słynnych mebli z PRL; Stary Fotel – Krzesła Bumerang metamorfoza</t>
-  </si>
-  <si>
-    <t>łukowato wygięte przednie nogi w kształcie bumerangu; gięte boczne elementy drewniane; tapicerowane prostokątne siedzisko; tapicerowane oparcie; smukła lekka bryła; cienki drewniany stelaż; zwężające się ku dołowi nogi; wyraźny prześwit pod siedziskiem; organiczny profil boczny; lekko odchylone oparcie; minimalistyczna forma lat 60.; charakterystyczna sylwetka bumerangu</t>
-  </si>
-  <si>
-    <t>Typ 300-227</t>
-  </si>
-  <si>
-    <t>Celia</t>
-  </si>
-  <si>
-    <t>ok. 1965; produkcja na przełomie lat 60. i 70. XX w.</t>
-  </si>
-  <si>
-    <t>Zamojskie Fabryki Mebli</t>
-  </si>
-  <si>
-    <t>brak podłokietników; toczone drewniane nogi umieszczone po bokach części tapicerowanej; trapezowe siedzisko; proste tapicerowane oparcie; lekka minimalistyczna forma; kompaktowe wymiary; stylistyka skandynawskiego modernizmu</t>
-  </si>
-  <si>
-    <t>drewniany stelaż; toczone nogi; tapicerowane siedzisko; tapicerowane oparcie; otwarta konstrukcja bez podłokietników; konstrukcja szkieletowa przeznaczona do produkcji seryjnej</t>
-  </si>
-  <si>
-    <t>typ 300-190 Lisek; typ 366; GFM-64; lekkie fotele klubowe PRL bez podłokietników</t>
-  </si>
-  <si>
-    <t>fotele Zamojskich Fabryk Mebli z lat 60. i 70.; meble klubowe produkowane w Zamościu; modele o minimalistycznej konstrukcji bez podłokietników</t>
-  </si>
-  <si>
-    <t>Meblostan – Fotel CELIA typ 300-227; Patyna – Fotel CELIA typ 300-227 PRL; Szajba Sklep – Fotel Celia typ 300-227; materiały kolekcjonerskie dotyczące Zamojskich Fabryk Mebli</t>
-  </si>
-  <si>
-    <t>brak podłokietników; toczone drewniane nogi umieszczone po bokach korpusu; trapezowe tapicerowane siedzisko; prostokątne tapicerowane oparcie; lekka minimalistyczna bryła; duży prześwit pod siedziskiem; cienki drewniany stelaż; zwężające się ku dołowi nogi; odsłonięte drewniane elementy boczne; kompaktowe proporcje; geometryczny profil boczny; forma inspirowana skandynawskim modernizmem</t>
-  </si>
-  <si>
-    <t>Typ 300-139</t>
-  </si>
-  <si>
-    <t>Stefan</t>
-  </si>
-  <si>
-    <t>Swarzędzka Fabryka Mebli</t>
-  </si>
-  <si>
-    <t>szerokie drewniane podłokietniki o łagodnym łuku; otwarta konstrukcja boczna; luźne tapicerowane poduchy siedziska i oparcia; rozłożysta bryła; lekka skandynawska stylistyka; nisko osadzone siedzisko; masywny drewniany stelaż</t>
-  </si>
-  <si>
-    <t>stelaż z litego drewna bukowego; otwarta rama boczna; osobna poduszka siedziska; osobna poduszka oparcia; pasy tapicerskie; konstrukcja szkieletowa skręcana</t>
-  </si>
-  <si>
-    <t>typ 300-123 Puchała; typ 366; duńskie fotele Kandidaten projektu Ib Kofod-Larsena; fotele skandynawskie lat 60</t>
-  </si>
-  <si>
-    <t>sofa Stefan; zestawy wypoczynkowe Swarzędzkiej Fabryki Mebli; meble eksportowe Swarzędzkiej Fabryki Mebli z lat 60.</t>
-  </si>
-  <si>
-    <t>„Meble w produkcji 1962” – Zjednoczenie Przemysłu Meblarskiego; „Meble do małych mieszkań. Informator”, Wydawnictwo Katalogów i Cenników 1966; Laminerva – „Ikony polskiego designu: Fotel Stefan typ 300-139”; Meblostan – Para foteli Stefan typ 300-139; Patyna – Para foteli Stefan typ 300-139</t>
-  </si>
-  <si>
-    <t>szerokie wyprofilowane drewniane podłokietniki; otwarta drewniana rama boczna; luźna poduszka siedziska; luźna poduszka oparcia; nisko osadzone głębokie siedzisko; prostokątne grube poduchy; lekko odchylone oparcie; masywny bukowy stelaż; duży prześwit pod siedziskiem; szeroki rozstaw przednich nóg; profil boczny inspirowany wzornictwem skandynawskim; rozłożysta bryła eksportowa</t>
-  </si>
-  <si>
-    <t>B-3300</t>
-  </si>
-  <si>
-    <t>ok. 1969; produkcja w końcu lat 60. i na początku lat 70. XX w</t>
-  </si>
-  <si>
-    <t>Zakład Mebli Giętych w Radomsku; Fabryki Mebli Radomsko (późniejsze nazewnictwo zakładu)</t>
-  </si>
-  <si>
-    <t>gięte drewniane podłokietniki; szerokie tapicerowane siedzisko; prostokątne tapicerowane oparcie; otwarta konstrukcja boczna; gięty bukowy stelaż; nisko osadzona bryła; elegancka modernistyczna forma</t>
-  </si>
-  <si>
-    <t>stelaż z giętego drewna bukowego; tapicerowane siedzisko; tapicerowane oparcie; konstrukcja szkieletowa; elementy gięte wykonane w technologii Thoneta; konstrukcja skręcana</t>
-  </si>
-  <si>
-    <t>B-310 VAR; B-6028; GFM-64; typ 300-139 Stefan</t>
-  </si>
-  <si>
-    <t>fotele Zakładu Mebli Giętych w Radomsku; modele eksportowe Radomsko z lat 60. i 70.; rodzina foteli z giętego drewna bukowego</t>
-  </si>
-  <si>
-    <t>Patyna – Fotel B-3300 Zakład Mebli Giętych w Radomsku; Meblostan – Para foteli B-3300; archiwalne materiały Fabryk Mebli Radomsko; oferty kolekcjonerskie dokumentujące oryginalne oznaczenie modelu</t>
-  </si>
-  <si>
-    <t>gięte drewniane podłokietniki; otwarta drewniana rama boczna; szerokie prostokątne oparcie; szerokie głębokie siedzisko; bukowy gięty stelaż; duży prześwit pod siedziskiem; łagodnie wygięte boki; zwężające się ku dołowi nogi; lekko pochylone oparcie; masywniejsza bryła niż typ 366; widoczne elementy z giętego drewna; modernistyczna forma gabinetowa</t>
-  </si>
-  <si>
-    <t>Cechy AI</t>
   </si>
 </sst>
 </file>
@@ -4230,7 +4342,7 @@
         <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>103</v>
+        <v>294</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="381.75">
@@ -4238,7 +4350,7 @@
         <v>104</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>113</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="366">
@@ -4246,7 +4358,7 @@
         <v>26</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>123</v>
+        <v>296</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="91.5">
@@ -4262,7 +4374,7 @@
         <v>38</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>143</v>
+        <v>297</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="91.5">

</xml_diff>